<commit_message>
feat: pricing spreadsheet complete, expense spreadsheet updated
- Added all perfumes, deodorants & body mists to pricing spreadsheet
  (DEODORANTS MEN/WOMEN, PERFUMES MEN/WOMEN, BODY MIST — 73 new rows)
- Added scripts: fix-prices-correct-names.mjs, add-perfumes-deodorants-to-excel.mjs
- Expense spreadsheet: added Amazon MUNBYN printer order (May 8, $239.66)
- Moved receipt to processed folder

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis.xlsx
+++ b/AmericanSelect_PricingAnalysis.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC91E0DB-0EB2-4F56-A19B-7DC9BA1CC6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B5299E-8F6F-423A-A74A-231A23D47441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +13,8 @@
     <sheet name="Summary by Category" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pricing Analysis'!$A$1:$F$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pricing Analysis'!$A$1:$F$246</definedName>
+    <definedName name="_xlnm._FilterDatabase">'Pricing Analysis'!$A$1:$F$173</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="288">
   <si>
     <t>STATUS</t>
   </si>
@@ -643,6 +644,240 @@
   </si>
   <si>
     <t>45W Type-C Charger Super Fast Charging - White</t>
+  </si>
+  <si>
+    <t>DEODORANTS (MEN)</t>
+  </si>
+  <si>
+    <t>Degree Men Black + White Ultraclear Deodorant</t>
+  </si>
+  <si>
+    <t>AXE Antiperspirant Deodorant for Men Essence, 48H Sweat &amp; Odor Protection, Black Pepper &amp; Cedarwood</t>
+  </si>
+  <si>
+    <t>AXE Apollo Antiperspirant Deodorant Stick For Men, Sage &amp; Cedarwood, 48 Hr Anti Sweat</t>
+  </si>
+  <si>
+    <t>Right Guard Sport Fresh Scent Antiperspirant &amp; Deodorant Invisible Solid 4-in-1 For Men, 48-Hour Odor Protection</t>
+  </si>
+  <si>
+    <t>DEODORANTS (WOMEN)</t>
+  </si>
+  <si>
+    <t>Lady Speed Stick 72HR Antiperspirant Deodorant for Women, Invisible Dry, Shower Fresh Scent, 2.3 oz</t>
+  </si>
+  <si>
+    <t>Suave Antiperspirant Deodorant For Women, 48hr Protection, Fresh</t>
+  </si>
+  <si>
+    <t>Suave Antiperspirant Deodorant For Women, 48hr Protection, Powder</t>
+  </si>
+  <si>
+    <t>Suave Antiperspirant Deodorant For Women, Wild Cherry Blossom</t>
+  </si>
+  <si>
+    <t>Suave Antiperspirant Deodorant For Women, 48hr Protection, Tropical Paradise</t>
+  </si>
+  <si>
+    <t>Degree Original Antiperspirant Deodorant Sheer Powder</t>
+  </si>
+  <si>
+    <t>PERFUMES (MEN)</t>
+  </si>
+  <si>
+    <t>Taj Max Aqua Sport 3.4 oz Long-Lasting Perfume</t>
+  </si>
+  <si>
+    <t>Taj Max Exotic Bliss 3.4 oz Long-Lasting Perfume</t>
+  </si>
+  <si>
+    <t>Loveryblack Affinity For Him Pheromone Cologne</t>
+  </si>
+  <si>
+    <t>Loveryblack Affinity At Midnight Pheromone Perfume (Unisex)</t>
+  </si>
+  <si>
+    <t>Loveryblack Affinity Pure Passion Pheromone Perfume (Unisex)</t>
+  </si>
+  <si>
+    <t>Mens Cologne Bross 3.4oz Eau De Parfum Spray, Masculine Mist</t>
+  </si>
+  <si>
+    <t>Men'S Extreme 3.4oz Eau De Parfum - Men Perfume Spray</t>
+  </si>
+  <si>
+    <t>Victorious Heroes Spray Cologne Eau De Toilette For Men</t>
+  </si>
+  <si>
+    <t>Adventure Club Perfume For Men</t>
+  </si>
+  <si>
+    <t>Azure Vantage Aqua Spray Cologne Eau De Parfum For Men</t>
+  </si>
+  <si>
+    <t>Investor Gold Spray Cologne Eau De Parfum For Men</t>
+  </si>
+  <si>
+    <t>Invincible Black Spray Cologne For Men EDP</t>
+  </si>
+  <si>
+    <t>Invincible Platinum Spray Cologne Eau De Toilette For Men</t>
+  </si>
+  <si>
+    <t>Magic Code Spray Cologne Eau De Toilette For Men</t>
+  </si>
+  <si>
+    <t>Prism Cologne Eau De Toilette For Men</t>
+  </si>
+  <si>
+    <t>Daspar De Homme Men Perfume with Pheromones</t>
+  </si>
+  <si>
+    <t>PERFUMES (WOMEN)</t>
+  </si>
+  <si>
+    <t>Charm Spray Perfume Eau De Parfum For Women</t>
+  </si>
+  <si>
+    <t>Daicy Blue Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Flower Pink Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Gorgeous Flower Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Honey Bear Pink Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Love Is Forever Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Nice Girl Spray Perfume Eau De Parfum For Women</t>
+  </si>
+  <si>
+    <t>Princess High Heels Pink Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Sexy Rose Pink Spray Perfume Eau De Parfum</t>
+  </si>
+  <si>
+    <t>365 Day Spray Perfume Eau De Parfum For Women</t>
+  </si>
+  <si>
+    <t>Paris Night Just for Men</t>
+  </si>
+  <si>
+    <t>Infinity 3.3 oz EDT For Men</t>
+  </si>
+  <si>
+    <t>Platinum 3.4 oz EDP For Men</t>
+  </si>
+  <si>
+    <t>Savage 3.4 oz EDP For Men</t>
+  </si>
+  <si>
+    <t>Victory 3.3 oz EDT For Men</t>
+  </si>
+  <si>
+    <t>Hercules Paris 3.4 oz EDP For Men</t>
+  </si>
+  <si>
+    <t>Men'S Salvang 3.4oz Eau De Parfume</t>
+  </si>
+  <si>
+    <t>Bleu De Rivoli Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Blue Intense Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Eau De Vivre Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Imperial Oud Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Legende Intense Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Reverie Pour Homme Eau De Parfum</t>
+  </si>
+  <si>
+    <t>Fantastic Pink 3.4 oz EDP For Women</t>
+  </si>
+  <si>
+    <t>Fleur De Paris 3.4 oz EDP For Women</t>
+  </si>
+  <si>
+    <t>Lazell Night Bloom For Women EDP 3.4 oz</t>
+  </si>
+  <si>
+    <t>Lazell Spring For Women EDP 3.4 oz</t>
+  </si>
+  <si>
+    <t>Miss Coco 3.4 oz EDP For Women</t>
+  </si>
+  <si>
+    <t>Flower Eau De Parfum For Women</t>
+  </si>
+  <si>
+    <t>Lazell Black Onyx Women EDP 3.4</t>
+  </si>
+  <si>
+    <t>Harmonie De Jour Eau De Parfum</t>
+  </si>
+  <si>
+    <t>BODY MIST</t>
+  </si>
+  <si>
+    <t>Island Coconut Body Mist</t>
+  </si>
+  <si>
+    <t>Passion Fruit Body Mist</t>
+  </si>
+  <si>
+    <t>Watermelon Sugar Body Mist</t>
+  </si>
+  <si>
+    <t>Pineapple Dream Body Mist</t>
+  </si>
+  <si>
+    <t>So Fresh La Vanille Angel Cake Body Mist - Vanilla Marshmallow</t>
+  </si>
+  <si>
+    <t>So Fresh La Vanille Angel Cake Body Mist - Vanilla Coconut</t>
+  </si>
+  <si>
+    <t>So Fresh La Vanille Angel Cake Body Mist - Vanilla Ice Cream</t>
+  </si>
+  <si>
+    <t>So Fresh The Beaches Collection Let's Get Away Body Mist - South Beach</t>
+  </si>
+  <si>
+    <t>So Fresh The Beaches Collection Let's Get Away Body Mist - Copacabana Beach</t>
+  </si>
+  <si>
+    <t>So Fresh The Beaches Collection Let's Get Away Body Mist - Maui Beach</t>
+  </si>
+  <si>
+    <t>So Fresh The Dulce Collection Utopia Body Mist - Red Velvet</t>
+  </si>
+  <si>
+    <t>So Fresh The Dulce Collection Utopia Body Mist - Chocolate Dreams</t>
+  </si>
+  <si>
+    <t>So Fresh The Dulce Collection Utopia Body Mist - Cherry On Top</t>
+  </si>
+  <si>
+    <t>So Fresh Wildflower Collection Morning Dew Body Mist - Forget Me Not</t>
+  </si>
+  <si>
+    <t>So Fresh Wildflower Collection Morning Dew Body Mist - Sunset Blossom</t>
+  </si>
+  <si>
+    <t>So Fresh Wildflower Collection Morning Dew Body Mist - Desert Willow</t>
   </si>
   <si>
     <t># Items</t>
@@ -665,7 +900,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="#,##0\ &quot;XAF&quot;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -687,12 +922,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -724,11 +953,38 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color rgb="FF4A0070"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF4A0070"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -807,6 +1063,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFE0B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9F9F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1BEE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFBBDEFB"/>
       </patternFill>
     </fill>
@@ -828,16 +1109,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCEDC8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE0B2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
     <fill>
@@ -899,7 +1170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -928,13 +1199,13 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -943,22 +1214,22 @@
     <xf numFmtId="165" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -967,22 +1238,136 @@
     <xf numFmtId="165" fontId="0" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -994,19 +1379,43 @@
     <xf numFmtId="165" fontId="0" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="26" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="26" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1016,90 +1425,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1442,13 +1767,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1464,7 +1789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1472,7 +1797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1522,15 +1847,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:F173"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F246"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="58" customWidth="1"/>
@@ -1539,7 +1863,7 @@
     <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>18</v>
       </c>
@@ -1559,7 +1883,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>24</v>
       </c>
@@ -1579,7 +1903,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>24</v>
       </c>
@@ -1599,7 +1923,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>24</v>
       </c>
@@ -1619,7 +1943,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
@@ -1639,7 +1963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>24</v>
       </c>
@@ -1659,7 +1983,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>24</v>
       </c>
@@ -1679,7 +2003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>24</v>
       </c>
@@ -1699,7 +2023,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>24</v>
       </c>
@@ -1719,7 +2043,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>24</v>
       </c>
@@ -1739,7 +2063,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>24</v>
       </c>
@@ -1759,7 +2083,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>24</v>
       </c>
@@ -1779,7 +2103,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>24</v>
       </c>
@@ -1799,7 +2123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>24</v>
       </c>
@@ -1819,7 +2143,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>24</v>
       </c>
@@ -1839,7 +2163,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
@@ -1859,7 +2183,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>24</v>
       </c>
@@ -1879,7 +2203,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>24</v>
       </c>
@@ -1899,7 +2223,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>24</v>
       </c>
@@ -1919,7 +2243,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>24</v>
       </c>
@@ -1939,7 +2263,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>24</v>
       </c>
@@ -1959,7 +2283,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>24</v>
       </c>
@@ -1979,7 +2303,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>24</v>
       </c>
@@ -1999,7 +2323,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>24</v>
       </c>
@@ -2019,7 +2343,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>24</v>
       </c>
@@ -2039,7 +2363,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>49</v>
       </c>
@@ -2059,7 +2383,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>49</v>
       </c>
@@ -2079,7 +2403,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>49</v>
       </c>
@@ -2099,7 +2423,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>49</v>
       </c>
@@ -2119,7 +2443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>49</v>
       </c>
@@ -2139,7 +2463,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>49</v>
       </c>
@@ -2159,7 +2483,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>49</v>
       </c>
@@ -2179,7 +2503,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>49</v>
       </c>
@@ -2199,7 +2523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>49</v>
       </c>
@@ -2219,7 +2543,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>49</v>
       </c>
@@ -2239,7 +2563,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>49</v>
       </c>
@@ -2259,7 +2583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>49</v>
       </c>
@@ -2279,7 +2603,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>49</v>
       </c>
@@ -2299,7 +2623,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>49</v>
       </c>
@@ -2319,7 +2643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>49</v>
       </c>
@@ -2339,7 +2663,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>49</v>
       </c>
@@ -2359,7 +2683,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>49</v>
       </c>
@@ -2379,7 +2703,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>49</v>
       </c>
@@ -2399,7 +2723,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>49</v>
       </c>
@@ -2419,7 +2743,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>49</v>
       </c>
@@ -2439,7 +2763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>49</v>
       </c>
@@ -2459,7 +2783,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>49</v>
       </c>
@@ -2479,7 +2803,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>49</v>
       </c>
@@ -2499,7 +2823,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>49</v>
       </c>
@@ -2519,7 +2843,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>49</v>
       </c>
@@ -2539,7 +2863,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>49</v>
       </c>
@@ -2559,7 +2883,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>49</v>
       </c>
@@ -2579,7 +2903,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>49</v>
       </c>
@@ -2599,7 +2923,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>49</v>
       </c>
@@ -2619,7 +2943,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>49</v>
       </c>
@@ -2639,7 +2963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>49</v>
       </c>
@@ -2659,7 +2983,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>49</v>
       </c>
@@ -2679,7 +3003,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>49</v>
       </c>
@@ -2699,7 +3023,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>49</v>
       </c>
@@ -2719,7 +3043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>49</v>
       </c>
@@ -2739,7 +3063,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>85</v>
       </c>
@@ -2759,7 +3083,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>85</v>
       </c>
@@ -2779,7 +3103,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>85</v>
       </c>
@@ -2793,13 +3117,13 @@
         <v>4500</v>
       </c>
       <c r="E63" s="15">
-        <v>6500</v>
+        <v>5500</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>85</v>
       </c>
@@ -2819,7 +3143,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>85</v>
       </c>
@@ -2839,7 +3163,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>91</v>
       </c>
@@ -2859,7 +3183,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>91</v>
       </c>
@@ -2879,7 +3203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>91</v>
       </c>
@@ -2899,7 +3223,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>91</v>
       </c>
@@ -2919,7 +3243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>91</v>
       </c>
@@ -2939,7 +3263,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>91</v>
       </c>
@@ -2959,7 +3283,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>91</v>
       </c>
@@ -2979,7 +3303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>91</v>
       </c>
@@ -2999,7 +3323,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>91</v>
       </c>
@@ -3019,7 +3343,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>91</v>
       </c>
@@ -3039,7 +3363,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>91</v>
       </c>
@@ -3059,7 +3383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>91</v>
       </c>
@@ -3079,7 +3403,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>91</v>
       </c>
@@ -3099,7 +3423,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>91</v>
       </c>
@@ -3119,7 +3443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>91</v>
       </c>
@@ -3139,7 +3463,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>91</v>
       </c>
@@ -3159,7 +3483,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>91</v>
       </c>
@@ -3179,7 +3503,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>91</v>
       </c>
@@ -3199,7 +3523,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>110</v>
       </c>
@@ -3219,7 +3543,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>110</v>
       </c>
@@ -3239,7 +3563,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>110</v>
       </c>
@@ -3259,7 +3583,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>110</v>
       </c>
@@ -3279,7 +3603,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>110</v>
       </c>
@@ -3299,7 +3623,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>116</v>
       </c>
@@ -3319,7 +3643,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>116</v>
       </c>
@@ -3339,7 +3663,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>116</v>
       </c>
@@ -3359,7 +3683,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>116</v>
       </c>
@@ -3379,7 +3703,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>116</v>
       </c>
@@ -3399,7 +3723,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>122</v>
       </c>
@@ -3419,7 +3743,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>122</v>
       </c>
@@ -3439,7 +3763,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>122</v>
       </c>
@@ -3459,7 +3783,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>122</v>
       </c>
@@ -3479,7 +3803,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>122</v>
       </c>
@@ -3499,7 +3823,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>122</v>
       </c>
@@ -3519,7 +3843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>122</v>
       </c>
@@ -3539,7 +3863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>122</v>
       </c>
@@ -3559,7 +3883,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>122</v>
       </c>
@@ -3579,7 +3903,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>122</v>
       </c>
@@ -3599,7 +3923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>122</v>
       </c>
@@ -3619,7 +3943,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>122</v>
       </c>
@@ -3639,7 +3963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>135</v>
       </c>
@@ -3659,7 +3983,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>135</v>
       </c>
@@ -3679,7 +4003,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
         <v>135</v>
       </c>
@@ -3699,7 +4023,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
         <v>135</v>
       </c>
@@ -3719,7 +4043,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
         <v>135</v>
       </c>
@@ -3739,7 +4063,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>135</v>
       </c>
@@ -3759,7 +4083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
         <v>135</v>
       </c>
@@ -3779,7 +4103,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
         <v>135</v>
       </c>
@@ -3799,7 +4123,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
         <v>135</v>
       </c>
@@ -3819,7 +4143,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>135</v>
       </c>
@@ -3839,7 +4163,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>135</v>
       </c>
@@ -3859,7 +4183,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>135</v>
       </c>
@@ -3879,7 +4203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>135</v>
       </c>
@@ -3899,7 +4223,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>135</v>
       </c>
@@ -3919,7 +4243,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>135</v>
       </c>
@@ -3939,7 +4263,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>135</v>
       </c>
@@ -3959,7 +4283,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>135</v>
       </c>
@@ -3979,7 +4303,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>135</v>
       </c>
@@ -3999,7 +4323,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>135</v>
       </c>
@@ -4019,7 +4343,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>135</v>
       </c>
@@ -4039,7 +4363,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>135</v>
       </c>
@@ -4059,7 +4383,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>135</v>
       </c>
@@ -4079,7 +4403,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>135</v>
       </c>
@@ -4099,7 +4423,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>135</v>
       </c>
@@ -4119,7 +4443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>135</v>
       </c>
@@ -4139,7 +4463,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>135</v>
       </c>
@@ -4159,7 +4483,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>135</v>
       </c>
@@ -4179,7 +4503,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>135</v>
       </c>
@@ -4199,7 +4523,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
         <v>135</v>
       </c>
@@ -4219,7 +4543,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
         <v>135</v>
       </c>
@@ -4239,7 +4563,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
         <v>135</v>
       </c>
@@ -4259,7 +4583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
         <v>135</v>
       </c>
@@ -4279,7 +4603,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
         <v>135</v>
       </c>
@@ -4299,7 +4623,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
         <v>135</v>
       </c>
@@ -4319,7 +4643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
         <v>135</v>
       </c>
@@ -4339,7 +4663,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
         <v>135</v>
       </c>
@@ -4359,7 +4683,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
         <v>135</v>
       </c>
@@ -4379,7 +4703,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
         <v>135</v>
       </c>
@@ -4399,7 +4723,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
         <v>135</v>
       </c>
@@ -4419,7 +4743,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>135</v>
       </c>
@@ -4439,7 +4763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>135</v>
       </c>
@@ -4459,7 +4783,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
         <v>135</v>
       </c>
@@ -4479,7 +4803,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
         <v>135</v>
       </c>
@@ -4499,7 +4823,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="149" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
         <v>135</v>
       </c>
@@ -4519,7 +4843,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
         <v>135</v>
       </c>
@@ -4539,7 +4863,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
         <v>135</v>
       </c>
@@ -4559,7 +4883,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
         <v>135</v>
       </c>
@@ -4579,7 +4903,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="153" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
         <v>135</v>
       </c>
@@ -4599,7 +4923,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
         <v>135</v>
       </c>
@@ -4619,7 +4943,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
         <v>135</v>
       </c>
@@ -4639,7 +4963,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="156" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
         <v>135</v>
       </c>
@@ -4659,7 +4983,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
         <v>135</v>
       </c>
@@ -4679,7 +5003,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="158" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
         <v>135</v>
       </c>
@@ -4699,7 +5023,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
         <v>135</v>
       </c>
@@ -4719,7 +5043,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="160" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
         <v>135</v>
       </c>
@@ -4739,7 +5063,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
         <v>135</v>
       </c>
@@ -4759,7 +5083,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
         <v>135</v>
       </c>
@@ -4779,7 +5103,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="163" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
         <v>135</v>
       </c>
@@ -4793,13 +5117,13 @@
         <v>4000</v>
       </c>
       <c r="E163" s="15">
-        <v>12000</v>
+        <v>5000</v>
       </c>
       <c r="F163" s="16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
         <v>135</v>
       </c>
@@ -4819,7 +5143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="165" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
         <v>195</v>
       </c>
@@ -4839,7 +5163,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
         <v>195</v>
       </c>
@@ -4859,7 +5183,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
         <v>195</v>
       </c>
@@ -4879,7 +5203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="168" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
         <v>195</v>
       </c>
@@ -4899,7 +5223,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="169" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
         <v>200</v>
       </c>
@@ -4919,7 +5243,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="170" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
         <v>200</v>
       </c>
@@ -4939,7 +5263,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="171" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
         <v>200</v>
       </c>
@@ -4959,7 +5283,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="172" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
         <v>200</v>
       </c>
@@ -4979,7 +5303,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
         <v>200</v>
       </c>
@@ -4999,23 +5323,1477 @@
         <v>12</v>
       </c>
     </row>
+    <row r="174" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B174" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="C174" s="29">
+        <v>4.5</v>
+      </c>
+      <c r="D174" s="30">
+        <v>3000</v>
+      </c>
+      <c r="E174" s="15">
+        <v>3000</v>
+      </c>
+      <c r="F174" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B175" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="C175" s="29">
+        <v>5</v>
+      </c>
+      <c r="D175" s="30">
+        <v>3000</v>
+      </c>
+      <c r="E175" s="15">
+        <v>3000</v>
+      </c>
+      <c r="F175" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B176" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="C176" s="29">
+        <v>5</v>
+      </c>
+      <c r="D176" s="30">
+        <v>3000</v>
+      </c>
+      <c r="E176" s="15">
+        <v>3000</v>
+      </c>
+      <c r="F176" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B177" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="C177" s="29">
+        <v>4</v>
+      </c>
+      <c r="D177" s="30">
+        <v>2000</v>
+      </c>
+      <c r="E177" s="15">
+        <v>2000</v>
+      </c>
+      <c r="F177" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B178" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="C178" s="21">
+        <v>3.5</v>
+      </c>
+      <c r="D178" s="22">
+        <v>1500</v>
+      </c>
+      <c r="E178" s="15">
+        <v>1500</v>
+      </c>
+      <c r="F178" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B179" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="C179" s="21">
+        <v>3</v>
+      </c>
+      <c r="D179" s="22">
+        <v>2300</v>
+      </c>
+      <c r="E179" s="15">
+        <v>2300</v>
+      </c>
+      <c r="F179" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B180" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C180" s="21">
+        <v>3</v>
+      </c>
+      <c r="D180" s="22">
+        <v>2300</v>
+      </c>
+      <c r="E180" s="15">
+        <v>2300</v>
+      </c>
+      <c r="F180" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B181" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="C181" s="21">
+        <v>3</v>
+      </c>
+      <c r="D181" s="22">
+        <v>2300</v>
+      </c>
+      <c r="E181" s="15">
+        <v>2300</v>
+      </c>
+      <c r="F181" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B182" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="C182" s="21">
+        <v>3</v>
+      </c>
+      <c r="D182" s="22">
+        <v>2300</v>
+      </c>
+      <c r="E182" s="15">
+        <v>2300</v>
+      </c>
+      <c r="F182" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B183" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="C183" s="21">
+        <v>4.5</v>
+      </c>
+      <c r="D183" s="22">
+        <v>3200</v>
+      </c>
+      <c r="E183" s="15">
+        <v>3200</v>
+      </c>
+      <c r="F183" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B184" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="C184" s="29">
+        <v>15</v>
+      </c>
+      <c r="D184" s="30">
+        <v>12000</v>
+      </c>
+      <c r="E184" s="15">
+        <v>12000</v>
+      </c>
+      <c r="F184" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B185" s="28" t="s">
+        <v>220</v>
+      </c>
+      <c r="C185" s="29">
+        <v>15</v>
+      </c>
+      <c r="D185" s="30">
+        <v>12000</v>
+      </c>
+      <c r="E185" s="15">
+        <v>12000</v>
+      </c>
+      <c r="F185" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B186" s="28" t="s">
+        <v>221</v>
+      </c>
+      <c r="C186" s="29">
+        <v>12</v>
+      </c>
+      <c r="D186" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E186" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F186" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B187" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="C187" s="29">
+        <v>12</v>
+      </c>
+      <c r="D187" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E187" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F187" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B188" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="C188" s="29">
+        <v>12</v>
+      </c>
+      <c r="D188" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E188" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F188" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B189" s="28" t="s">
+        <v>224</v>
+      </c>
+      <c r="C189" s="29">
+        <v>12</v>
+      </c>
+      <c r="D189" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E189" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F189" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B190" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="C190" s="29">
+        <v>12</v>
+      </c>
+      <c r="D190" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E190" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F190" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B191" s="28" t="s">
+        <v>226</v>
+      </c>
+      <c r="C191" s="29">
+        <v>10</v>
+      </c>
+      <c r="D191" s="30">
+        <v>6000</v>
+      </c>
+      <c r="E191" s="15">
+        <v>6000</v>
+      </c>
+      <c r="F191" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B192" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="C192" s="29">
+        <v>10</v>
+      </c>
+      <c r="D192" s="30">
+        <v>7000</v>
+      </c>
+      <c r="E192" s="15">
+        <v>7000</v>
+      </c>
+      <c r="F192" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B193" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="C193" s="29">
+        <v>8</v>
+      </c>
+      <c r="D193" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E193" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F193" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B194" s="28" t="s">
+        <v>229</v>
+      </c>
+      <c r="C194" s="29">
+        <v>8</v>
+      </c>
+      <c r="D194" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E194" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F194" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B195" s="28" t="s">
+        <v>230</v>
+      </c>
+      <c r="C195" s="29">
+        <v>8</v>
+      </c>
+      <c r="D195" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E195" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F195" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B196" s="28" t="s">
+        <v>231</v>
+      </c>
+      <c r="C196" s="29">
+        <v>8</v>
+      </c>
+      <c r="D196" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E196" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F196" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B197" s="28" t="s">
+        <v>232</v>
+      </c>
+      <c r="C197" s="29">
+        <v>8</v>
+      </c>
+      <c r="D197" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E197" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F197" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B198" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="C198" s="29">
+        <v>8</v>
+      </c>
+      <c r="D198" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E198" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F198" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B199" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="C199" s="29">
+        <v>5</v>
+      </c>
+      <c r="D199" s="30">
+        <v>4000</v>
+      </c>
+      <c r="E199" s="15">
+        <v>4000</v>
+      </c>
+      <c r="F199" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B200" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="C200" s="21">
+        <v>12</v>
+      </c>
+      <c r="D200" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E200" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F200" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B201" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="C201" s="21">
+        <v>12</v>
+      </c>
+      <c r="D201" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E201" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F201" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B202" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="C202" s="21">
+        <v>12</v>
+      </c>
+      <c r="D202" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E202" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F202" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B203" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="C203" s="21">
+        <v>12</v>
+      </c>
+      <c r="D203" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E203" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F203" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B204" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="C204" s="21">
+        <v>12</v>
+      </c>
+      <c r="D204" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E204" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F204" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B205" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="C205" s="21">
+        <v>12</v>
+      </c>
+      <c r="D205" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E205" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F205" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B206" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="C206" s="21">
+        <v>12</v>
+      </c>
+      <c r="D206" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E206" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F206" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B207" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="C207" s="21">
+        <v>12</v>
+      </c>
+      <c r="D207" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E207" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F207" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B208" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="C208" s="21">
+        <v>12</v>
+      </c>
+      <c r="D208" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E208" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F208" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="B209" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="C209" s="21">
+        <v>8</v>
+      </c>
+      <c r="D209" s="22">
+        <v>6500</v>
+      </c>
+      <c r="E209" s="15">
+        <v>6500</v>
+      </c>
+      <c r="F209" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B210" s="35" t="s">
+        <v>246</v>
+      </c>
+      <c r="C210" s="29">
+        <v>5</v>
+      </c>
+      <c r="D210" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E210" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F210" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B211" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="C211" s="29">
+        <v>5</v>
+      </c>
+      <c r="D211" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E211" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F211" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B212" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="C212" s="29">
+        <v>5</v>
+      </c>
+      <c r="D212" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E212" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F212" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A213" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B213" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="C213" s="29">
+        <v>5</v>
+      </c>
+      <c r="D213" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E213" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F213" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A214" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B214" s="35" t="s">
+        <v>250</v>
+      </c>
+      <c r="C214" s="29">
+        <v>5</v>
+      </c>
+      <c r="D214" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E214" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F214" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B215" s="35" t="s">
+        <v>251</v>
+      </c>
+      <c r="C215" s="29">
+        <v>5</v>
+      </c>
+      <c r="D215" s="30">
+        <v>5000</v>
+      </c>
+      <c r="E215" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F215" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B216" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="C216" s="29">
+        <v>10</v>
+      </c>
+      <c r="D216" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E216" s="36">
+        <v>10000</v>
+      </c>
+      <c r="F216" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B217" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="C217" s="29">
+        <v>15</v>
+      </c>
+      <c r="D217" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E217" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F217" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B218" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="C218" s="29">
+        <v>15</v>
+      </c>
+      <c r="D218" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E218" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F218" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B219" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="C219" s="29">
+        <v>15</v>
+      </c>
+      <c r="D219" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E219" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F219" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A220" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B220" s="35" t="s">
+        <v>256</v>
+      </c>
+      <c r="C220" s="29">
+        <v>15</v>
+      </c>
+      <c r="D220" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E220" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F220" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A221" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B221" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="C221" s="29">
+        <v>15</v>
+      </c>
+      <c r="D221" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E221" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F221" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A222" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="B222" s="35" t="s">
+        <v>258</v>
+      </c>
+      <c r="C222" s="29">
+        <v>15</v>
+      </c>
+      <c r="D222" s="30">
+        <v>15000</v>
+      </c>
+      <c r="E222" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F222" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A223" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B223" s="39" t="s">
+        <v>259</v>
+      </c>
+      <c r="C223" s="21">
+        <v>5</v>
+      </c>
+      <c r="D223" s="22">
+        <v>5000</v>
+      </c>
+      <c r="E223" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F223" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A224" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B224" s="39" t="s">
+        <v>260</v>
+      </c>
+      <c r="C224" s="21">
+        <v>8</v>
+      </c>
+      <c r="D224" s="22">
+        <v>8000</v>
+      </c>
+      <c r="E224" s="36">
+        <v>8000</v>
+      </c>
+      <c r="F224" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A225" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B225" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="C225" s="21">
+        <v>8</v>
+      </c>
+      <c r="D225" s="22">
+        <v>8000</v>
+      </c>
+      <c r="E225" s="36">
+        <v>8000</v>
+      </c>
+      <c r="F225" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A226" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B226" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="C226" s="21">
+        <v>8</v>
+      </c>
+      <c r="D226" s="22">
+        <v>8000</v>
+      </c>
+      <c r="E226" s="36">
+        <v>8000</v>
+      </c>
+      <c r="F226" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A227" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B227" s="39" t="s">
+        <v>263</v>
+      </c>
+      <c r="C227" s="21">
+        <v>5</v>
+      </c>
+      <c r="D227" s="22">
+        <v>5000</v>
+      </c>
+      <c r="E227" s="36">
+        <v>5000</v>
+      </c>
+      <c r="F227" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A228" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B228" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="C228" s="21">
+        <v>10</v>
+      </c>
+      <c r="D228" s="22">
+        <v>10000</v>
+      </c>
+      <c r="E228" s="36">
+        <v>10000</v>
+      </c>
+      <c r="F228" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A229" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B229" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="C229" s="21">
+        <v>8</v>
+      </c>
+      <c r="D229" s="22">
+        <v>8000</v>
+      </c>
+      <c r="E229" s="36">
+        <v>8000</v>
+      </c>
+      <c r="F229" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A230" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="B230" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="C230" s="21">
+        <v>15</v>
+      </c>
+      <c r="D230" s="22">
+        <v>15000</v>
+      </c>
+      <c r="E230" s="36">
+        <v>15000</v>
+      </c>
+      <c r="F230" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A231" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B231" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="C231" s="29">
+        <v>3</v>
+      </c>
+      <c r="D231" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E231" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F231" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A232" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B232" s="35" t="s">
+        <v>269</v>
+      </c>
+      <c r="C232" s="29">
+        <v>3</v>
+      </c>
+      <c r="D232" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E232" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F232" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A233" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B233" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="C233" s="29">
+        <v>3</v>
+      </c>
+      <c r="D233" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E233" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F233" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A234" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B234" s="35" t="s">
+        <v>271</v>
+      </c>
+      <c r="C234" s="29">
+        <v>3</v>
+      </c>
+      <c r="D234" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E234" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F234" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A235" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B235" s="35" t="s">
+        <v>272</v>
+      </c>
+      <c r="C235" s="29">
+        <v>3</v>
+      </c>
+      <c r="D235" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E235" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F235" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A236" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B236" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="C236" s="29">
+        <v>3</v>
+      </c>
+      <c r="D236" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E236" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F236" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A237" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B237" s="35" t="s">
+        <v>274</v>
+      </c>
+      <c r="C237" s="29">
+        <v>3</v>
+      </c>
+      <c r="D237" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E237" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F237" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A238" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B238" s="35" t="s">
+        <v>275</v>
+      </c>
+      <c r="C238" s="29">
+        <v>3</v>
+      </c>
+      <c r="D238" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E238" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F238" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A239" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B239" s="35" t="s">
+        <v>276</v>
+      </c>
+      <c r="C239" s="29">
+        <v>3</v>
+      </c>
+      <c r="D239" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E239" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F239" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A240" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B240" s="35" t="s">
+        <v>277</v>
+      </c>
+      <c r="C240" s="29">
+        <v>3</v>
+      </c>
+      <c r="D240" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E240" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F240" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A241" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B241" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="C241" s="29">
+        <v>3</v>
+      </c>
+      <c r="D241" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E241" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F241" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A242" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B242" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="C242" s="29">
+        <v>3</v>
+      </c>
+      <c r="D242" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E242" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F242" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="243" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A243" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B243" s="35" t="s">
+        <v>280</v>
+      </c>
+      <c r="C243" s="29">
+        <v>3</v>
+      </c>
+      <c r="D243" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E243" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F243" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="244" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A244" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B244" s="35" t="s">
+        <v>281</v>
+      </c>
+      <c r="C244" s="29">
+        <v>3</v>
+      </c>
+      <c r="D244" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E244" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F244" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A245" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B245" s="35" t="s">
+        <v>282</v>
+      </c>
+      <c r="C245" s="29">
+        <v>3</v>
+      </c>
+      <c r="D245" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E245" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F245" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A246" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="B246" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="C246" s="29">
+        <v>3</v>
+      </c>
+      <c r="D246" s="30">
+        <v>3500</v>
+      </c>
+      <c r="E246" s="36">
+        <v>3500</v>
+      </c>
+      <c r="F246" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F173" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="BODY LOTION"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F246" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -5024,195 +6802,263 @@
     <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="41" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1" s="41" t="s">
+        <v>285</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="41" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="43">
+        <v>24</v>
+      </c>
+      <c r="C2" s="44">
+        <v>4.93</v>
+      </c>
+      <c r="D2" s="45">
+        <v>4200</v>
+      </c>
+      <c r="E2" s="45">
+        <v>7208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="47">
+        <v>35</v>
+      </c>
+      <c r="C3" s="48">
+        <v>7.46</v>
+      </c>
+      <c r="D3" s="49">
+        <v>6857</v>
+      </c>
+      <c r="E3" s="49">
+        <v>11186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="51">
+        <v>5</v>
+      </c>
+      <c r="C4" s="52">
+        <v>11.5</v>
+      </c>
+      <c r="D4" s="53">
+        <v>7400</v>
+      </c>
+      <c r="E4" s="53">
+        <v>17200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="54" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="55">
+        <v>18</v>
+      </c>
+      <c r="C5" s="56">
+        <v>6.47</v>
+      </c>
+      <c r="D5" s="57">
+        <v>6639</v>
+      </c>
+      <c r="E5" s="57">
+        <v>9556</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="58" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="59">
+        <v>5</v>
+      </c>
+      <c r="C6" s="60">
+        <v>8</v>
+      </c>
+      <c r="D6" s="61">
+        <v>6000</v>
+      </c>
+      <c r="E6" s="61">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="62" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="63">
+        <v>5</v>
+      </c>
+      <c r="C7" s="64">
+        <v>11.18</v>
+      </c>
+      <c r="D7" s="65">
+        <v>4600</v>
+      </c>
+      <c r="E7" s="65">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" s="67">
+        <v>12</v>
+      </c>
+      <c r="C8" s="68">
+        <v>16.25</v>
+      </c>
+      <c r="D8" s="69">
+        <v>8167</v>
+      </c>
+      <c r="E8" s="69">
+        <v>24375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="70" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="71">
+        <v>59</v>
+      </c>
+      <c r="C9" s="72">
+        <v>25.85</v>
+      </c>
+      <c r="D9" s="73">
+        <v>7051</v>
+      </c>
+      <c r="E9" s="73">
+        <v>38771</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="74" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" s="75">
+        <v>4</v>
+      </c>
+      <c r="C10" s="76">
+        <v>28</v>
+      </c>
+      <c r="D10" s="77">
+        <v>10750</v>
+      </c>
+      <c r="E10" s="77">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="78" t="s">
+        <v>200</v>
+      </c>
+      <c r="B11" s="79">
+        <v>5</v>
+      </c>
+      <c r="C11" s="80">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="D11" s="81">
+        <v>2000</v>
+      </c>
+      <c r="E11" s="81">
+        <v>15300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="66" t="s">
         <v>206</v>
       </c>
-      <c r="C1" s="27" t="s">
-        <v>207</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="29">
-        <v>24</v>
-      </c>
-      <c r="C2" s="30">
-        <v>4.93</v>
-      </c>
-      <c r="D2" s="31">
-        <v>4200</v>
-      </c>
-      <c r="E2" s="31">
-        <v>7208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="33">
-        <v>35</v>
-      </c>
-      <c r="C3" s="34">
-        <v>7.46</v>
-      </c>
-      <c r="D3" s="35">
-        <v>6857</v>
-      </c>
-      <c r="E3" s="35">
-        <v>11186</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="B4" s="37">
-        <v>5</v>
-      </c>
-      <c r="C4" s="38">
-        <v>11.5</v>
-      </c>
-      <c r="D4" s="39">
-        <v>7400</v>
-      </c>
-      <c r="E4" s="39">
-        <v>17200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="41">
-        <v>18</v>
-      </c>
-      <c r="C5" s="42">
-        <v>6.47</v>
-      </c>
-      <c r="D5" s="43">
-        <v>6639</v>
-      </c>
-      <c r="E5" s="43">
-        <v>9556</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="B6" s="45">
-        <v>5</v>
-      </c>
-      <c r="C6" s="46">
-        <v>8</v>
-      </c>
-      <c r="D6" s="47">
-        <v>6000</v>
-      </c>
-      <c r="E6" s="47">
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B7" s="49">
-        <v>5</v>
-      </c>
-      <c r="C7" s="50">
-        <v>11.18</v>
-      </c>
-      <c r="D7" s="51">
-        <v>4600</v>
-      </c>
-      <c r="E7" s="51">
-        <v>16800</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="52" t="s">
-        <v>122</v>
-      </c>
-      <c r="B8" s="53">
-        <v>12</v>
-      </c>
-      <c r="C8" s="54">
-        <v>16.25</v>
-      </c>
-      <c r="D8" s="55">
-        <v>8167</v>
-      </c>
-      <c r="E8" s="55">
-        <v>24375</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="56" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="57">
-        <v>59</v>
-      </c>
-      <c r="C9" s="58">
-        <v>25.85</v>
-      </c>
-      <c r="D9" s="59">
-        <v>7051</v>
-      </c>
-      <c r="E9" s="59">
-        <v>38771</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="60" t="s">
-        <v>195</v>
-      </c>
-      <c r="B10" s="61">
+      <c r="B12" s="67">
         <v>4</v>
       </c>
-      <c r="C10" s="62">
-        <v>28</v>
-      </c>
-      <c r="D10" s="63">
-        <v>10750</v>
-      </c>
-      <c r="E10" s="63">
-        <v>42000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="64" t="s">
-        <v>200</v>
-      </c>
-      <c r="B11" s="65">
-        <v>5</v>
-      </c>
-      <c r="C11" s="66">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="D11" s="67">
-        <v>2000</v>
-      </c>
-      <c r="E11" s="67">
-        <v>15300</v>
+      <c r="C12" s="68">
+        <v>4.63</v>
+      </c>
+      <c r="D12" s="69">
+        <v>2750</v>
+      </c>
+      <c r="E12" s="69">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="62" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" s="63">
+        <v>6</v>
+      </c>
+      <c r="C13" s="64">
+        <v>3.33</v>
+      </c>
+      <c r="D13" s="65">
+        <v>2317</v>
+      </c>
+      <c r="E13" s="65">
+        <v>2317</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="82" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="83">
+        <v>16</v>
+      </c>
+      <c r="C14" s="84">
+        <v>10.19</v>
+      </c>
+      <c r="D14" s="85">
+        <v>7563</v>
+      </c>
+      <c r="E14" s="85">
+        <v>7563</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="70" t="s">
+        <v>235</v>
+      </c>
+      <c r="B15" s="71">
+        <v>10</v>
+      </c>
+      <c r="C15" s="72">
+        <v>11.6</v>
+      </c>
+      <c r="D15" s="73">
+        <v>9650</v>
+      </c>
+      <c r="E15" s="73">
+        <v>9650</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update pricing & expense spreadsheets, add profit analysis script
- AmericanSelect_PricingAnalysis.xlsx: updated with perfumes, deodorants, body mists
- receipts/American_Select_Expenses.xlsx: MUNBYN printer expense added, totals corrected
- scripts/profit-analysis.mjs: ROI calculator comparing live prices vs expenses

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis.xlsx
+++ b/AmericanSelect_PricingAnalysis.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B5299E-8F6F-423A-A74A-231A23D47441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5006818A-70A1-440F-82A4-0C7350EF7257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3203,7 +3203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="11" t="s">
         <v>91</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="11" t="s">
         <v>91</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="11" t="s">
         <v>91</v>
       </c>
@@ -3263,7 +3263,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>91</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="11" t="s">
         <v>91</v>
       </c>
@@ -5583,7 +5583,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" s="32" t="s">
         <v>218</v>
       </c>
@@ -5603,7 +5603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" s="32" t="s">
         <v>218</v>
       </c>
@@ -5623,7 +5623,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" s="32" t="s">
         <v>218</v>
       </c>
@@ -5643,7 +5643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" s="32" t="s">
         <v>218</v>
       </c>
@@ -5663,7 +5663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" s="32" t="s">
         <v>218</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" s="32" t="s">
         <v>218</v>
       </c>
@@ -5703,7 +5703,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" s="32" t="s">
         <v>218</v>
       </c>
@@ -5723,7 +5723,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="194" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" s="32" t="s">
         <v>218</v>
       </c>
@@ -5743,7 +5743,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" s="32" t="s">
         <v>218</v>
       </c>
@@ -5763,7 +5763,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" s="32" t="s">
         <v>218</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A197" s="32" t="s">
         <v>218</v>
       </c>
@@ -5803,7 +5803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198" s="32" t="s">
         <v>218</v>
       </c>
@@ -5823,7 +5823,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A199" s="32" t="s">
         <v>218</v>
       </c>
@@ -5843,7 +5843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200" s="33" t="s">
         <v>235</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="201" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A201" s="33" t="s">
         <v>235</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="202" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A202" s="33" t="s">
         <v>235</v>
       </c>
@@ -5903,7 +5903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A203" s="33" t="s">
         <v>235</v>
       </c>
@@ -5923,7 +5923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A204" s="33" t="s">
         <v>235</v>
       </c>
@@ -5943,7 +5943,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A205" s="33" t="s">
         <v>235</v>
       </c>
@@ -5963,7 +5963,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A206" s="33" t="s">
         <v>235</v>
       </c>
@@ -5983,7 +5983,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A207" s="33" t="s">
         <v>235</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A208" s="33" t="s">
         <v>235</v>
       </c>
@@ -6023,7 +6023,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A209" s="33" t="s">
         <v>235</v>
       </c>
@@ -6043,7 +6043,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A210" s="34" t="s">
         <v>218</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A211" s="34" t="s">
         <v>218</v>
       </c>
@@ -6083,7 +6083,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A212" s="34" t="s">
         <v>218</v>
       </c>
@@ -6103,7 +6103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A213" s="34" t="s">
         <v>218</v>
       </c>
@@ -6123,7 +6123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A214" s="34" t="s">
         <v>218</v>
       </c>
@@ -6143,7 +6143,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A215" s="34" t="s">
         <v>218</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A216" s="34" t="s">
         <v>218</v>
       </c>
@@ -6183,7 +6183,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A217" s="34" t="s">
         <v>218</v>
       </c>
@@ -6203,7 +6203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A218" s="34" t="s">
         <v>218</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A219" s="34" t="s">
         <v>218</v>
       </c>

</xml_diff>

<commit_message>
fix: update all 157 shortened product names in pricing spreadsheet to exact names
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis.xlsx
+++ b/AmericanSelect_PricingAnalysis.xlsx
@@ -1,27 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5006818A-70A1-440F-82A4-0C7350EF7257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Legend" sheetId="1" r:id="rId1"/>
-    <sheet name="Pricing Analysis" sheetId="2" r:id="rId2"/>
-    <sheet name="Summary by Category" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Legend" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Pricing Analysis" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Summary by Category" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pricing Analysis'!$A$1:$F$246</definedName>
     <definedName name="_xlnm._FilterDatabase">'Pricing Analysis'!$A$1:$F$173</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -103,184 +96,184 @@
     <t>BODY WASH</t>
   </si>
   <si>
-    <t>Dr Teal's Body Wash - Prebiotic Lemon Balm 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Eucalyptus Spearmint 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Vanilla Comfort 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Hawaiian Bliss 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Soothe &amp; Sleep Lavender 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Coconut Oil 24oz</t>
-  </si>
-  <si>
-    <t>Dr Teal's Body Wash - Shea Butter &amp; Almond 24oz</t>
-  </si>
-  <si>
-    <t>Olay Essential Botanicals - Spiced Chai &amp; Pear</t>
-  </si>
-  <si>
-    <t>Olay Essential Botanicals - White Tea &amp; Cucumber</t>
-  </si>
-  <si>
-    <t>Olay Essential Botanicals - Lavender Milk &amp; Sandalwood</t>
-  </si>
-  <si>
-    <t>Suave Men Hydrating 3-in-1 Body Hair Face Wash 18oz</t>
-  </si>
-  <si>
-    <t>Suave Moisturizing Body Wash - Cocoa Butter &amp; Shea 18oz</t>
-  </si>
-  <si>
-    <t>Suave Cocoa Butter + Shea Body Wash 30oz</t>
-  </si>
-  <si>
-    <t>Suave Moisturizing Body Wash - Sweet Pea &amp; Violet 18oz</t>
-  </si>
-  <si>
-    <t>Suave Ocean Breeze Body Wash 18oz</t>
-  </si>
-  <si>
-    <t>Suave Ocean Breeze Body Wash 30oz</t>
-  </si>
-  <si>
-    <t>Suave Wild Cherry Blossom Body Wash 30oz</t>
-  </si>
-  <si>
-    <t>Suave Strawberry Delight Body Wash 30oz</t>
-  </si>
-  <si>
-    <t>Suave Milk &amp; Honey Body Wash 30oz</t>
-  </si>
-  <si>
-    <t>NIVEA MEN Maximum Hydration 3-in-1 Body Wash</t>
+    <t>Dr Teal's Body Wash with Prebiotic Lemon Balm and Essential Oil Blend</t>
+  </si>
+  <si>
+    <t>Dr Teal's Body Wash Relax and Relief with Eucalyptus Spearmint</t>
+  </si>
+  <si>
+    <t>Dr Teal's Vanilla Comfort Body Wash with Pure Epsom Salt</t>
+  </si>
+  <si>
+    <t>Dr Teal's Hawaiian Bliss Body Wash with Alaea Red Sea Salt, Hibiscus &amp; Papaya, 24 fl oz</t>
+  </si>
+  <si>
+    <t>Dr Teal's Body Wash with Pure Epsom Salt, Soothe &amp; Sleep with Lavender</t>
+  </si>
+  <si>
+    <t>Dr Teal's Body Wash, Nourish &amp; Protect with Coconut Oil</t>
+  </si>
+  <si>
+    <t>Dr Teal's Body Wash with Pure Epsom Salt, Shea Butter &amp; Almond</t>
+  </si>
+  <si>
+    <t>Olay Essential Botanicals Body Wash, Spiced Chai &amp; Pear</t>
+  </si>
+  <si>
+    <t>Olay Essential Botanicals Body Wash, White Tea &amp; Cucumber</t>
+  </si>
+  <si>
+    <t>Olay Essential Botanicals Body Wash, Lavender Milk &amp; Sandalwood</t>
+  </si>
+  <si>
+    <t>Suave Men Hydrating 3-in-1 Body, Hair &amp; Face Wash with Glycerin &amp; Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Moisturizing Body Wash Cocoa Butter and Shea with Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Cocoa Butter + Shea Moisturizing Body Wash with Glycerin &amp; Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Moisturizing Body Wash Sweet Pea &amp; Violet with Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Ocean Breeze Moisturizing Body Wash with Glycerin &amp; Vitamin E, 18 fl oz</t>
+  </si>
+  <si>
+    <t>Suave Ocean Breeze Moisturizing Body Wash with Glycerin &amp; Vitamin E, 30 fl oz</t>
+  </si>
+  <si>
+    <t>Suave Wild Cherry Blossom Moisturizing Body Wash with Glycerin &amp; Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Strawberry Delight Moisturizing Body Wash with Glycerin &amp; Vitamin E</t>
+  </si>
+  <si>
+    <t>Suave Milk &amp; Honey Moisturizing Body Wash with Glycerin &amp; Vitamin E</t>
+  </si>
+  <si>
+    <t>NIVEA MEN Maximum Hydration 3-in-1 Body Wash with Aloe Vera</t>
   </si>
   <si>
     <t>Irish Spring Original Clean Deodorant Bar Soap</t>
   </si>
   <si>
-    <t>St. Ives Body Wash - Pink Lemon &amp; Mandarin Orange 22oz</t>
-  </si>
-  <si>
-    <t>St. Ives Body Wash - Sea Salt &amp; Pacific Kelp 22oz</t>
-  </si>
-  <si>
-    <t>St. Ives Body Wash - Oatmeal &amp; Shea Butter 22oz</t>
+    <t>St. Ives Body Wash Pink Lemon and Mandarin Orange</t>
+  </si>
+  <si>
+    <t>St. Ives Sea Salt &amp; Pacific Kelp Exfoliating Body Wash</t>
+  </si>
+  <si>
+    <t>St. Ives Soothing Body Wash, Oatmeal &amp; Shea Butter, 22 fl oz</t>
   </si>
   <si>
     <t>BODY LOTION</t>
   </si>
   <si>
-    <t>Olay Body Lotion - Age Defying with Niacinamide Serum</t>
-  </si>
-  <si>
-    <t>Olay Body Lotion - Nourishing with Hyaluronic Acid Serum</t>
-  </si>
-  <si>
-    <t>Olay Body Lotion - Smoothing with Retinol Serum</t>
-  </si>
-  <si>
-    <t>Olay Body Lotion - Tone Enhancing with AHA Serum</t>
+    <t>Olay Body Lotion Age Defying with Niacinamide Serum</t>
+  </si>
+  <si>
+    <t>Olay Body Lotion Nourishing with Hyaluronic Acid Serum</t>
+  </si>
+  <si>
+    <t>Olay Body Lotion Smoothing with Retinol Serum</t>
+  </si>
+  <si>
+    <t>Olay Body Lotion Tone Enhancing with AHA Serum</t>
   </si>
   <si>
     <t>Aveeno Daily Moisturizing Body Lotion 18oz</t>
   </si>
   <si>
-    <t>Jergens Hydrating Coconut Body Lotion</t>
-  </si>
-  <si>
-    <t>Jergens Shea Butter Hand and Body Lotion</t>
-  </si>
-  <si>
-    <t>Jergens Soothing Aloe Body Lotion</t>
-  </si>
-  <si>
-    <t>Jergens Skin Firming Body Lotion with Collagen &amp; Elastin</t>
-  </si>
-  <si>
-    <t>Jergens Ultra Healing Dry Skin Lotion</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture+ Body Lotion - Prebiotic Lemon Balm</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture+ Body Lotion - Eucalyptus &amp; Spearmint</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture+ Body Lotion - Coconut Oil</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture+ Body Lotion - Shea Butter &amp; Almond</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture Body Lotion - Lavender</t>
-  </si>
-  <si>
-    <t>Dr Teal's 24hr Moisture Body Lotion - Vanilla Comfort</t>
-  </si>
-  <si>
-    <t>Vaseline Men Cooling Hydration 3-in-1 Lotion with Menthol</t>
-  </si>
-  <si>
-    <t>Vaseline Men Fast Absorbing 3-in-1 Lotion</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Cocoa Radiant</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Soothing Hydration Aloe Vera</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Sensitive Skin Relief Oatmeal</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Calm Healing Lavender</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Unscented Advanced Repair</t>
-  </si>
-  <si>
-    <t>Vaseline Intensive Care - Nourishing Moisture Oat Extract</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Coconut &amp; Orchid</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Sweet Almond Oil</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Oatmeal &amp; Shea Butter</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Collagen &amp; Elastin with Pump</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Rose &amp; Argan Oil</t>
-  </si>
-  <si>
-    <t>St. Ives Hand &amp; Body Lotion - Vitamin E &amp; Avocado Oil</t>
-  </si>
-  <si>
-    <t>Cetaphil Face &amp; Body Moisturizing Lotion (all skin types)</t>
-  </si>
-  <si>
-    <t>CeraVe Daily Moisturizing Face &amp; Body Lotion (Normal to Dry)</t>
-  </si>
-  <si>
-    <t>CeraVe Moisturizing Cream (Normal to Very Dry)</t>
-  </si>
-  <si>
-    <t>Lubriderm Fragrance Free Daily Moisture Lotion (large)</t>
-  </si>
-  <si>
-    <t>Lubriderm Daily Moisture Lotion 6oz</t>
+    <t>Jergens Hydrating Coconut Body Lotion, Hand and Body Moisturizer, Infused with Coconut Oil</t>
+  </si>
+  <si>
+    <t>Jergens Shea Butter Hand and Body Lotion, Deep Conditioning Moisturizer</t>
+  </si>
+  <si>
+    <t>Jergens Soothing Aloe Body Lotion, Aloe Vera Body and Hand Moisturizer</t>
+  </si>
+  <si>
+    <t>Jergens Skin Firming Body Lotion with Collagen and Elastin</t>
+  </si>
+  <si>
+    <t>Jergens Ultra Healing Dry Skin Lotion, Hand and Body Moisturizer</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture+ Body Lotion, Prebiotic Lemon Balm &amp; Essential Oils</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture+ Body Lotion, Eucalyptus &amp; Spearmint</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture+ Body Lotion, Coconut Oil &amp; Essential Oils</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture+ Body Lotion, Shea Butter &amp; Almond</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture Body Lotion with Lavender Essential Oil</t>
+  </si>
+  <si>
+    <t>Dr Teal's 24 Hour Moisture Body Lotion, Vanilla Comfort</t>
+  </si>
+  <si>
+    <t>Vaseline Men Cooling Hydration 3-in-1 Face, Hands &amp; Body Lotion with Menthol</t>
+  </si>
+  <si>
+    <t>Vaseline Men Fast Absorbing 3-in-1 Face, Hands &amp; Body Lotion For Men, For Dry Skin, Absorbs in Just 15 Seconds for Moisturized Skin</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Body Lotion Cocoa Radiant with Pure Cocoa Butter</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Soothing Hydration Body Lotion with Aloe Vera</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Sensitive Skin Relief Body Lotion with Colloidal Oatmeal</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Calm Healing Body Lotion with Lavender Extract</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Unscented Advanced Repair Body Lotion</t>
+  </si>
+  <si>
+    <t>Vaseline Intensive Care Nourishing Moisture Body Lotion with Pure Oat Extract</t>
+  </si>
+  <si>
+    <t>St. Ives Coconut &amp; Orchid Hand &amp; Body Lotion, Softening Body Care for Dry Skin</t>
+  </si>
+  <si>
+    <t>St. Ives Hand &amp; Body Lotion, Sweet Almond Oil, Restoring Body Care for Dry Skin</t>
+  </si>
+  <si>
+    <t>St. Ives Oatmeal &amp; Shea Butter Hand &amp; Body Lotion, Moisturizing Body Care for Dry Skin</t>
+  </si>
+  <si>
+    <t>St. Ives Renewing Hand &amp; Body Lotion with Pump, Daily Moisturizer Collagen Elastin for Dry Skin, Made with 100% Natural Moisturizers</t>
+  </si>
+  <si>
+    <t>St. Ives Rose &amp; Argan Oil Hand &amp; Body Lotion, Smoothing Body Care for Dry Skin</t>
+  </si>
+  <si>
+    <t>St. Ives Vitamin E &amp; Avocado Oil Hand &amp; Body Lotion, Hydrating Body Care for Dry Skin</t>
+  </si>
+  <si>
+    <t>Cetaphil Face &amp; Body Moisturizer, Hydrating Moisturizing Lotion for All Skin Types, Suitable for Sensitive Skin</t>
+  </si>
+  <si>
+    <t>CeraVe Daily Moisturizing Face &amp; Body Lotion for Normal to Dry Skin</t>
+  </si>
+  <si>
+    <t>CeraVe Moisturizing Cream for Face &amp; Body Normal to Very Dry Skin</t>
+  </si>
+  <si>
+    <t>Lubriderm Fragrance Free Daily Moisture Lotion + Pro-Ceramide, Shea Butter &amp; Glycerin, Face, Hand &amp; Body Lotion for Sensitive Skin, Hydrating Lotion for Healthier-Looking Skin</t>
+  </si>
+  <si>
+    <t>Lubriderm Daily Moisture Lotion + Pro-Ceramide, Shea Butter &amp; Glycerin, Hydrating Face, Hand &amp; Body Lotion, 24-hour Moisturizer for Dry Skin, 6 Fl Oz</t>
   </si>
   <si>
     <t>PERSONAL CARE</t>
@@ -292,310 +285,310 @@
     <t>Crest Pro-Health Advanced Mouthwash</t>
   </si>
   <si>
-    <t>Nair Body Cream Hair Removal Cream</t>
-  </si>
-  <si>
-    <t>Men's Electric Shaver 3-in-1 USB Rechargeable</t>
-  </si>
-  <si>
-    <t>LQT Men's Electric Shaver (Exquisite Box / USB Charging)</t>
+    <t>Nair Body Cream, Hair Removal Cream</t>
+  </si>
+  <si>
+    <t>Men's Electric Shaver 3 in 1 - Portable USB Rechargeable Shaver Featuring 3D Floating Blades and a Digital Display Suitable for Both Wet and Dry Shaving</t>
+  </si>
+  <si>
+    <t>LQT Men's Electric Shaver | Exquisite Packaging Box, USB Charging, Lithium Battery, Matte Texture, Essential for Men, Beard Trimming</t>
   </si>
   <si>
     <t>HAIR</t>
   </si>
   <si>
-    <t>Suave Keratin Infusion Smoothing Shampoo &amp; Conditioner Set</t>
-  </si>
-  <si>
-    <t>Suave Moisturizing Shampoo &amp; Conditioner - Almond &amp; Shea Butter</t>
-  </si>
-  <si>
-    <t>TRESemmé Rich Moisture Shampoo &amp; Conditioner Set (28oz each)</t>
-  </si>
-  <si>
-    <t>TRESemmé Keratin Smooth Shampoo &amp; Conditioner Set</t>
-  </si>
-  <si>
-    <t>TRESemmé Anti-Breakage Shampoo &amp; Conditioner Set</t>
-  </si>
-  <si>
-    <t>TRESemmé Amplified Volume Shampoo &amp; Conditioner Set</t>
-  </si>
-  <si>
-    <t>TRESemmé Silky &amp; Smooth Anti-Frizz Shampoo &amp; Conditioner Set</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Silver Blonde</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Dark Blonde</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Radiant Raspberry</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Auburn Brown</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Burgundy</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Bright Auburn</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Vibrant Violet</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Deep Burgundy</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Brown Black</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Black</t>
-  </si>
-  <si>
-    <t>Revlon ColorSilk Permanent Hair Color - Ultra Light Ash Blonde</t>
+    <t>Suave Keratin Infusion Smoothing Shampoo &amp; Conditioner Set For Frizzy Hair</t>
+  </si>
+  <si>
+    <t>Suave Moisturizing Shampoo &amp; Conditioner With Almond &amp; Shea Butter</t>
+  </si>
+  <si>
+    <t>TRESemmé Rich Moisture Shampoo and Conditioner Set</t>
+  </si>
+  <si>
+    <t>TRESemmé Shampoo &amp; Conditioner Keratin Smooth</t>
+  </si>
+  <si>
+    <t>TRESemmé Shampoo And Conditioner Anti-Breakage</t>
+  </si>
+  <si>
+    <t>TRESemmé Shampoo and Conditioner for Women Amplified Volume Twin Pack</t>
+  </si>
+  <si>
+    <t>TRESemmé Silky &amp; Smooth Anti-Frizz Shampoo &amp; Conditioner for Frizzy Hair</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Silver Blonde)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Dark Blonde)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Radiant Raspberry)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Auburn Brown)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Burgundy)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Bright Auburn)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Vibrant Violet)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Deep Burgundy)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Brown Black)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Black)</t>
+  </si>
+  <si>
+    <t>Revlon ColorSilk Permanent Hair Color with Bond Repair Complex (Ultra Light Ash Blonde)</t>
   </si>
   <si>
     <t>KIDS &amp; BABY</t>
   </si>
   <si>
-    <t>Dr Teal's Kids 3-in-1 Sleep Bath - Melatonin &amp; Essential Oil</t>
-  </si>
-  <si>
-    <t>Dr Teal's Kids 3-in-1 Bubble Bath - Ashwagandha</t>
-  </si>
-  <si>
-    <t>Suave Kids Paw Patrol 3-in-1 Shampoo Conditioner Body Wash</t>
-  </si>
-  <si>
-    <t>Cetaphil Baby Daily Lotion with Organic Calendula</t>
-  </si>
-  <si>
-    <t>CeraVe Baby Lotion with Ceramides Niacinamide &amp; Vitamin E</t>
+    <t>Dr Teal's Kids 3-in-1 Sleep Bath: Bubble Bath, Body Wash &amp; Shampoo with Melatonin &amp; Essential Oil</t>
+  </si>
+  <si>
+    <t>Dr Teal's Kids 3-in-1 Bubble Bath, Body Wash &amp; Shampoo with Ashwagandha</t>
+  </si>
+  <si>
+    <t>Suave Kids Paw Patrol 3-in-1 Shampoo, Conditioner &amp; Body Wash, Adventure Bay Breeze</t>
+  </si>
+  <si>
+    <t>Cetaphil Baby Daily Lotion with Organic Calendula Vitamin E Sweet Almond &amp; Sunflower Oils</t>
+  </si>
+  <si>
+    <t>CeraVe Baby Lotion, Gentle Baby Skin Care with Ceramides, Niacinamide &amp; Vitamin E, Fragrance, Paraben, Dye &amp; Phthalates Free</t>
   </si>
   <si>
     <t>HOUSEHOLD</t>
   </si>
   <si>
-    <t>Febreze Air Freshener - Linen &amp; Sky 8.8oz</t>
-  </si>
-  <si>
-    <t>Febreze Air Mist - Heavy Duty Crisp Clean 8.8oz</t>
-  </si>
-  <si>
-    <t>Febreze Air Mist - Hawaiian Aloha 8.8oz</t>
-  </si>
-  <si>
-    <t>Febreze Air Effects - Mountain Scent 8.8oz</t>
-  </si>
-  <si>
-    <t>360 Spin Mop and Bucket Set with 4 Microfiber Refills</t>
+    <t>Febreze Air Freshener Spray, Odor-Fighting Room Spray, Linen &amp; Sky</t>
+  </si>
+  <si>
+    <t>Febreze Air Mist Air Freshener Spray, Heavy Duty Crisp Clean</t>
+  </si>
+  <si>
+    <t>Febreze Air Mist Air Freshener Spray Hawaiian Aloha</t>
+  </si>
+  <si>
+    <t>Febreze Air Effects Air Freshener - Mountain Scent</t>
+  </si>
+  <si>
+    <t>Mop and Bucket Set, 360° Spin Mop and Bucket Set and 4 Microfiber Mop Refills</t>
   </si>
   <si>
     <t>KITCHEN</t>
   </si>
   <si>
-    <t>Manual Pasta Maker Machine (9 Thickness Settings)</t>
-  </si>
-  <si>
-    <t>Reusable Stretchable Storage Lids (small set)</t>
-  </si>
-  <si>
-    <t>1000 Reusable Stretchable Storage Lids</t>
-  </si>
-  <si>
-    <t>Manual Food Chopper Pull String Vegetable &amp; Meat Mincer</t>
-  </si>
-  <si>
-    <t>Electric Mini Garlic Blender USB Rechargeable 8.45oz</t>
-  </si>
-  <si>
-    <t>380mL Rechargeable Portable Blender Cup - Green</t>
-  </si>
-  <si>
-    <t>380mL Rechargeable Portable Blender Cup - Black</t>
-  </si>
-  <si>
-    <t>380mL Rechargeable Portable Blender Cup - Pink</t>
-  </si>
-  <si>
-    <t>380mL Rechargeable Portable Blender Cup - Deep Purple</t>
-  </si>
-  <si>
-    <t>380mL Rechargeable Portable Blender Cup - Blue</t>
-  </si>
-  <si>
-    <t>Manual Chopper No Electricity - Pink</t>
-  </si>
-  <si>
-    <t>Manual Chopper No Electricity - Gray</t>
+    <t>Manual Pasta Maker Machine, 9 Adjustable Thickness Settings</t>
+  </si>
+  <si>
+    <t>Reusable Stretchable Storage Lids for Round Pots, Bowls, and Cups – Air-Tight, Food-Safe</t>
+  </si>
+  <si>
+    <t>1000 Reusable Stretchable Storage Lids for Round Pots, Bowls, and Cups – Air-Tight, Food-Safe</t>
+  </si>
+  <si>
+    <t>Manual Food Chopper, Pull String Vegetable and Meat Mincer with Clear Container, Hand-Powered Kitchen Processor</t>
+  </si>
+  <si>
+    <t>8.45oz RZSYZH USB Rechargeable Electric mini Garlic  Blender with Stainless Steel Blades for Automatic Chopping</t>
+  </si>
+  <si>
+    <t>380Ml Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender for Shakes And Smoothies, Juice (Green)</t>
+  </si>
+  <si>
+    <t>380Ml Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender for Shakes And Smoothies, Juice (Black)</t>
+  </si>
+  <si>
+    <t>380Ml Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender for Shakes And Smoothies, Juice (Pink)</t>
+  </si>
+  <si>
+    <t>380Ml Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender for Shakes And Smoothies, Juice (Deep Purple)</t>
+  </si>
+  <si>
+    <t>380Ml Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender for Shakes And Smoothies, Juice (Blue)</t>
+  </si>
+  <si>
+    <t>Manual Chopper. No Need for Electricity (Pink)</t>
+  </si>
+  <si>
+    <t>Manual Chopper. No Need for Electricity (Gray)</t>
   </si>
   <si>
     <t>ELECTRONICS</t>
   </si>
   <si>
-    <t>Smart Watch iPhone &amp; Android - Pink</t>
-  </si>
-  <si>
-    <t>Smart Watch iPhone &amp; Android - Black</t>
-  </si>
-  <si>
-    <t>Z68 Smartwatch (Wireless Calling / Sports) - Black</t>
-  </si>
-  <si>
-    <t>Z68 Smartwatch (Wireless Calling / Sports) - Gold</t>
-  </si>
-  <si>
-    <t>Z68 Smartwatch (Wireless Calling / Sports) - Pink</t>
-  </si>
-  <si>
-    <t>LAXASFIT Unisex Smartwatch (iPhone &amp; Android)</t>
-  </si>
-  <si>
-    <t>LAXASFIT Unisex Smartwatch - Black</t>
-  </si>
-  <si>
-    <t>PLEIVO Smartwatch 2.01in LED Flashlight Sports Tracker</t>
-  </si>
-  <si>
-    <t>PLEIVO Smartwatch 2.01in LED Flashlight - Black</t>
-  </si>
-  <si>
-    <t>Smart Watch Metal Frame Ceramic Base 2.01in Screen</t>
-  </si>
-  <si>
-    <t>Smart Watch Metal Frame Ceramic Base 2.01in Screen - Black</t>
-  </si>
-  <si>
-    <t>GT4 PRO Smartwatch Full Touchscreen 100+ Sports Modes</t>
-  </si>
-  <si>
-    <t>GT4 PRO Smartwatch Full Touchscreen 100+ Sports Modes - Black</t>
-  </si>
-  <si>
-    <t>Doviico 1.83in Smart Fitness Bracelet</t>
-  </si>
-  <si>
-    <t>Doviico 1.83in Smart Fitness Bracelet - Pink</t>
-  </si>
-  <si>
-    <t>256 GB Memory Card with Adapter</t>
+    <t>Smart Watch Compatible with iPhone &amp; Android Devices (Pink)</t>
+  </si>
+  <si>
+    <t>Smart Watch Compatible with iPhone &amp; Android Devices (Black)</t>
+  </si>
+  <si>
+    <t>Z68 Smartwatch Featuring Wireless Calling, Message Alerts, Various Sports Modes, Information Notifications, Multifunctional Phone Answering/Dialing, Remote Photography, Music Playback, Sports Tracking (Black)</t>
+  </si>
+  <si>
+    <t>Z68 Smartwatch Featuring Wireless Calling, Message Alerts, Various Sports Modes, Information Notifications, Multifunctional Phone Answering/Dialing, Remote Photography, Music Playback, Sports Tracking (Gold)</t>
+  </si>
+  <si>
+    <t>Z68 Smartwatch Featuring Wireless Calling, Message Alerts, Various Sports Modes, Information Notifications, Multifunctional Phone Answering/Dialing, Remote Photography, Music Playback, Sports Tracking (Pink)</t>
+  </si>
+  <si>
+    <t>LAXASFIT Unisex Smartwatch Compatible with Both iPhone and Android</t>
+  </si>
+  <si>
+    <t>LAXASFIT Unisex Smartwatch Compatible with Both iPhone and Android (Black)</t>
+  </si>
+  <si>
+    <t>PLEIVO New Smart Watch with 2.01-inch Large Screen, LED Flashlight, Outdoor Sports Watch, Fitness Tracker Compatible with Android and iPhone</t>
+  </si>
+  <si>
+    <t>PLEIVO New Smart Watch with 2.01-inch Large Screen, LED Flashlight, Outdoor Sports Watch, Fitness Tracker Compatible with Android and iPhone (Black)</t>
+  </si>
+  <si>
+    <t>Smart Watch with A Metal Frame, Ceramic Base, And A 2.01-inch Large Screen</t>
+  </si>
+  <si>
+    <t>Smart Watch with A Metal Frame, Ceramic Base, And A 2.01-inch Large Screen (Black)</t>
+  </si>
+  <si>
+    <t>GT4 PRO Smartwatch Featuring a Full Touchscreen, Wireless Calling, Over 100 Sports Modes, Weather Updates, Stopwatch, Timer, Alarm, SMS Notifications</t>
+  </si>
+  <si>
+    <t>GT4 PRO Smartwatch Featuring a Full Touchscreen, Wireless Calling, Over 100 Sports Modes, Weather Updates, Stopwatch, Timer, Alarm, SMS Notifications (Black)</t>
+  </si>
+  <si>
+    <t>Doviico 1.83-inch Touch Screen, Supports Call Function, Incoming Call And Message Notifications, Multifunctional Fitness And Sports Smart Bracelet, Wireless Connection with Android And Phones</t>
+  </si>
+  <si>
+    <t>Doviico 1.83-inch Touch Screen, Supports Call Function, Incoming Call And Message Notifications, Multifunctional Fitness And Sports Smart Bracelet, Wireless Connection with Android And Phones (Pink)</t>
+  </si>
+  <si>
+    <t>256 GB Memory Card with Adapter - Enough Storage for your data</t>
   </si>
   <si>
     <t>20000mAh Large-Capacity Mobile Power Bank</t>
   </si>
   <si>
-    <t>Rechargeable LED Torch / Flashlight High Power</t>
-  </si>
-  <si>
-    <t>Rechargeable Portable Fan - Purple</t>
-  </si>
-  <si>
-    <t>Rechargeable Portable Fan - Pink</t>
-  </si>
-  <si>
-    <t>Rechargeable Portable Fan - Black</t>
+    <t>Rechargeable LED Torch/Flashlight With High Power Lamp</t>
+  </si>
+  <si>
+    <t>Rechargeable Portable Fan (Purple)</t>
+  </si>
+  <si>
+    <t>Rechargeable Portable Fan (Pink)</t>
+  </si>
+  <si>
+    <t>Rechargeable Portable Fan (Black)</t>
   </si>
   <si>
     <t>Dark Grey USB Rechargeable Fan</t>
   </si>
   <si>
-    <t>Dark Grey USB Rechargeable Fan - Black</t>
-  </si>
-  <si>
-    <t>YISSVIC Electric Fly Swatter Foldable Bug Zapper</t>
-  </si>
-  <si>
-    <t>TG192 Outdoor Wireless Speaker 2400mAh - Green</t>
-  </si>
-  <si>
-    <t>TG192 Outdoor Wireless Speaker 2400mAh - Blue</t>
-  </si>
-  <si>
-    <t>TG192 Outdoor Wireless Speaker 2400mAh - Dark Red</t>
-  </si>
-  <si>
-    <t>TG192 Outdoor Wireless Speaker 2400mAh - Black</t>
-  </si>
-  <si>
-    <t>TG192 Outdoor Wireless Speaker 2400mAh - Army Green</t>
-  </si>
-  <si>
-    <t>TG537 Portable Wireless Speaker TWS - Blue</t>
-  </si>
-  <si>
-    <t>TG537 Portable Wireless Speaker TWS - Red</t>
-  </si>
-  <si>
-    <t>TG537 Portable Wireless Speaker TWS - Black</t>
-  </si>
-  <si>
-    <t>TG537 Portable Wireless Speaker TWS - Cyan</t>
-  </si>
-  <si>
-    <t>TG667 Compact Speaker (USB TF FM Radio) - Red</t>
-  </si>
-  <si>
-    <t>TG667 Compact Speaker (USB TF FM Radio) - Blue</t>
-  </si>
-  <si>
-    <t>TG667 Compact Speaker (USB TF FM Radio) - Black</t>
-  </si>
-  <si>
-    <t>TG667 Compact Speaker (USB TF FM Radio) - Purple</t>
-  </si>
-  <si>
-    <t>Portable Wireless Speaker 15W Stereo RGB Lighting</t>
-  </si>
-  <si>
-    <t>Hyundai LP5t Wireless Headphones Noise Cancellation - Gray</t>
-  </si>
-  <si>
-    <t>Hyundai LP5t Wireless Headphones Noise Cancellation - White</t>
-  </si>
-  <si>
-    <t>JS59 Wireless Headphones 4 ENC Mics HiFi 50hr USB-C</t>
-  </si>
-  <si>
-    <t>JS59 Wireless Headphones 4 ENC Mics HiFi 50hr USB-C - Black</t>
+    <t>Dark Grey USB Rechargeable Fan (Black)</t>
+  </si>
+  <si>
+    <t>YISSVIC Rechargeable Electric Fly Swatter Foldable Bug Zapper</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker (Green)</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker (Blue)</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker (Dark Red)</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker (Black)</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker (Army Green)</t>
+  </si>
+  <si>
+    <t>TG537 Portable Wireless Speaker - TWS Technology (Blue)</t>
+  </si>
+  <si>
+    <t>TG537 Portable Wireless Speaker - TWS Technology (Red)</t>
+  </si>
+  <si>
+    <t>TG537 Portable Wireless Speaker - TWS Technology (Black)</t>
+  </si>
+  <si>
+    <t>TG537 Portable Wireless Speaker - TWS Technology (Cyan)</t>
+  </si>
+  <si>
+    <t>TG667 Compact and Portable Wireless Speaker. It Supports USB, TF Cards, and FM Radio, and Can Connect to Mobile Phones, Tablets (Red)</t>
+  </si>
+  <si>
+    <t>TG667 Compact and Portable Wireless Speaker. It Supports USB, TF Cards, and FM Radio, and Can Connect to Mobile Phones, Tablets (Blue)</t>
+  </si>
+  <si>
+    <t>TG667 Compact and Portable Wireless Speaker. It Supports USB, TF Cards, and FM Radio, and Can Connect to Mobile Phones, Tablets (Black)</t>
+  </si>
+  <si>
+    <t>TG667 Compact and Portable Wireless Speaker. It Supports USB, TF Cards, and FM Radio, and Can Connect to Mobile Phones, Tablets (Purple)</t>
+  </si>
+  <si>
+    <t>Portable Wireless Speaker, 15W Stereo, RGB Lighting, Suitable for Both Indoor and Outdoor Use</t>
+  </si>
+  <si>
+    <t>Hyundai LP5t Wireless Headphones with Surround Sound and Noise Cancellation (Gray)</t>
+  </si>
+  <si>
+    <t>Hyundai LP5t Wireless Headphones with Surround Sound and Noise Cancellation (White)</t>
+  </si>
+  <si>
+    <t>JS59 Wireless Headphones, 5.4 Headphones with 4 ENC Noise-Cancelling Microphones, HiFi Stereo, 50 Hours of Playback Time, USB-C</t>
+  </si>
+  <si>
+    <t>JS59 Wireless Headphones, 5.4 Headphones with 4 ENC Noise-Cancelling Microphones, HiFi Stereo, 50 Hours of Playback Time, USB-C (Black)</t>
   </si>
   <si>
     <t>YD03 Wireless Earbuds</t>
   </si>
   <si>
-    <t>Airpod Pro (clone)</t>
-  </si>
-  <si>
-    <t>Monster Wireless Earbuds CVC 8.0 Noise Reduction</t>
-  </si>
-  <si>
-    <t>Acer OHR544 Wireless Headset Heavy Bass - Orange</t>
-  </si>
-  <si>
-    <t>Acer OHR544 Wireless Headset Heavy Bass - Beige</t>
-  </si>
-  <si>
-    <t>Acer OHR544 Wireless Headset Heavy Bass - Black</t>
-  </si>
-  <si>
-    <t>Ace OHR501 Wireless Headset Touch Control - Purple</t>
-  </si>
-  <si>
-    <t>Ace OHR501 Wireless Headset Touch Control - Black</t>
-  </si>
-  <si>
-    <t>Nokia Go Earbuds+ TWS-201 - White</t>
-  </si>
-  <si>
-    <t>Nokia Go Earbuds+ TWS-201 - Black</t>
-  </si>
-  <si>
-    <t>Wireless Earbuds with Charging Case USB-C TWS</t>
-  </si>
-  <si>
-    <t>Wireless Earbuds with Charging Case USB-C TWS - White</t>
+    <t>Airpod Pro</t>
+  </si>
+  <si>
+    <t>Monster Wireless Earbuds with CVC 8.0 Noise Reduction</t>
+  </si>
+  <si>
+    <t>Acer OHR544 Wireless Headset with Heavy Bass Stereo + Talking Noise Cancellation (Orange)</t>
+  </si>
+  <si>
+    <t>Acer OHR544 Wireless Headset with Heavy Bass Stereo + Talking Noise Cancellation (Beige)</t>
+  </si>
+  <si>
+    <t>Acer OHR544 Wireless Headset with Heavy Bass Stereo + Talking Noise Cancellation (Black)</t>
+  </si>
+  <si>
+    <t>Ace OHR501 Wireless 5.4 Bass Stereo Headset with Noise Cancelling Microphone, Touch Control (Purple)</t>
+  </si>
+  <si>
+    <t>Ace OHR501 Wireless 5.4 Bass Stereo Headset with Noise Cancelling Microphone, Touch Control (Black)</t>
+  </si>
+  <si>
+    <t>Nokia Go Earbuds+ TWS-201 (White)</t>
+  </si>
+  <si>
+    <t>Nokia Go Earbuds+ TWS-201 (Black)</t>
+  </si>
+  <si>
+    <t>Wireless Earbuds with Charging Case, USB Type-C Charging, TWS Technology</t>
+  </si>
+  <si>
+    <t>Wireless Earbuds with Charging Case, USB Type-C Charging, TWS Technology (White)</t>
   </si>
   <si>
     <t>Y01 Over the Ear Wireless Headphones</t>
@@ -604,10 +597,10 @@
     <t>TOZO T6 Wireless Earbuds IPX8 Waterproof</t>
   </si>
   <si>
-    <t>4-in-1 USB Mini SD Card Reader Dual Card Slots</t>
-  </si>
-  <si>
-    <t>USB 2.0 Type-C Flash Drive 128GB High-Speed</t>
+    <t>4-in-1 USB Mini SD Card Reader with Dual Card Slots</t>
+  </si>
+  <si>
+    <t>USB 2.0 Type-C Flash Drive 128GB High-Speed Memory Stick</t>
   </si>
   <si>
     <t>7-in-1 USB Extender Hub</t>
@@ -619,10 +612,10 @@
     <t>Non-Contact Forehead Digital Thermometer</t>
   </si>
   <si>
-    <t>Digital Wrist Blood Pressure Monitor Rechargeable LCD</t>
-  </si>
-  <si>
-    <t>Rechargeable Arm Blood Pressure Monitor Large LED Screen</t>
+    <t>Rechargeable/Battery Powered (Optional) Digital Wrist Blood Pressure Monitor with Large LCD, Voice Broadcast (Optional)</t>
+  </si>
+  <si>
+    <t>Rechargeable Arm Blood Pressure Monitor with Large LED Screen, Digital Blood Pressure Machine</t>
   </si>
   <si>
     <t>Rechargeable Digital Scale with USB Charging</t>
@@ -631,19 +624,19 @@
     <t>CABLES &amp; CHARGERS</t>
   </si>
   <si>
-    <t>Data Cable USB-C to USB-C Fast Charging</t>
-  </si>
-  <si>
-    <t>USB to USB-C Charging Cable</t>
+    <t>Data Cable, USB C to USB C Charging Cable, Type C to Type C Fast Charging</t>
+  </si>
+  <si>
+    <t>USB to USB C Charging Cable</t>
   </si>
   <si>
     <t>USB iPhone Charging Cable</t>
   </si>
   <si>
-    <t>45W Type-C Charger Super Fast Charging - Black</t>
-  </si>
-  <si>
-    <t>45W Type-C Charger Super Fast Charging - White</t>
+    <t>45W High Quality Type-C Charger - Super Fast Charging (Black)</t>
+  </si>
+  <si>
+    <t>45W High Quality Type-C Charger - Super Fast Charging (White)</t>
   </si>
   <si>
     <t>DEODORANTS (MEN)</t>
@@ -895,39 +888,39 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0\ &quot;XAF&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;XAF&quot;"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1A237E"/>
       <sz val="10"/>
-      <color rgb="FF1A237E"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -941,41 +934,20 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF4A0070"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF4A0070"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF4A0070"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1170,7 +1142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1271,31 +1243,13 @@
     <xf numFmtId="0" fontId="9" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1307,7 +1261,7 @@
     <xf numFmtId="165" fontId="0" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1319,7 +1273,7 @@
     <xf numFmtId="165" fontId="0" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1331,7 +1285,7 @@
     <xf numFmtId="165" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1343,7 +1297,7 @@
     <xf numFmtId="165" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1355,7 +1309,7 @@
     <xf numFmtId="165" fontId="0" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1367,7 +1321,7 @@
     <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1379,7 +1333,7 @@
     <xf numFmtId="165" fontId="0" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1391,7 +1345,7 @@
     <xf numFmtId="165" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1403,7 +1357,7 @@
     <xf numFmtId="165" fontId="0" fillId="26" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1415,7 +1369,7 @@
     <xf numFmtId="165" fontId="0" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1765,9 +1719,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -1781,7 +1735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1789,7 +1743,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1797,7 +1751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1805,7 +1759,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -1813,7 +1767,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1821,7 +1775,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -1829,7 +1783,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
@@ -1837,7 +1791,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
@@ -1847,14 +1801,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F246"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="58" customWidth="1"/>
@@ -1863,7 +1817,7 @@
     <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>18</v>
       </c>
@@ -1883,7 +1837,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>24</v>
       </c>
@@ -1903,7 +1857,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>24</v>
       </c>
@@ -1923,7 +1877,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>24</v>
       </c>
@@ -1943,7 +1897,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
@@ -1963,7 +1917,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>24</v>
       </c>
@@ -1983,7 +1937,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>24</v>
       </c>
@@ -2003,7 +1957,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>24</v>
       </c>
@@ -2023,7 +1977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>24</v>
       </c>
@@ -2043,7 +1997,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>24</v>
       </c>
@@ -2063,7 +2017,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>24</v>
       </c>
@@ -2083,7 +2037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>24</v>
       </c>
@@ -2103,7 +2057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>24</v>
       </c>
@@ -2123,7 +2077,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>24</v>
       </c>
@@ -2143,7 +2097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>24</v>
       </c>
@@ -2163,7 +2117,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
@@ -2183,7 +2137,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>24</v>
       </c>
@@ -2203,7 +2157,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>24</v>
       </c>
@@ -2223,7 +2177,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>24</v>
       </c>
@@ -2243,7 +2197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>24</v>
       </c>
@@ -2263,7 +2217,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>24</v>
       </c>
@@ -2283,7 +2237,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>24</v>
       </c>
@@ -2303,7 +2257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>24</v>
       </c>
@@ -2323,7 +2277,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>24</v>
       </c>
@@ -2343,7 +2297,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>24</v>
       </c>
@@ -2363,7 +2317,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>49</v>
       </c>
@@ -2383,7 +2337,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>49</v>
       </c>
@@ -2403,7 +2357,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>49</v>
       </c>
@@ -2423,7 +2377,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>49</v>
       </c>
@@ -2443,7 +2397,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>49</v>
       </c>
@@ -2463,7 +2417,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>49</v>
       </c>
@@ -2483,7 +2437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>49</v>
       </c>
@@ -2503,7 +2457,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>49</v>
       </c>
@@ -2523,7 +2477,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>49</v>
       </c>
@@ -2543,7 +2497,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>49</v>
       </c>
@@ -2563,7 +2517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>49</v>
       </c>
@@ -2583,7 +2537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>49</v>
       </c>
@@ -2603,7 +2557,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>49</v>
       </c>
@@ -2623,7 +2577,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>49</v>
       </c>
@@ -2643,7 +2597,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>49</v>
       </c>
@@ -2663,7 +2617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>49</v>
       </c>
@@ -2683,7 +2637,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>49</v>
       </c>
@@ -2703,7 +2657,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>49</v>
       </c>
@@ -2723,7 +2677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>49</v>
       </c>
@@ -2743,7 +2697,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>49</v>
       </c>
@@ -2763,7 +2717,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>49</v>
       </c>
@@ -2783,7 +2737,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>49</v>
       </c>
@@ -2803,7 +2757,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>49</v>
       </c>
@@ -2823,7 +2777,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>49</v>
       </c>
@@ -2843,7 +2797,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>49</v>
       </c>
@@ -2863,7 +2817,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>49</v>
       </c>
@@ -2883,7 +2837,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>49</v>
       </c>
@@ -2903,7 +2857,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>49</v>
       </c>
@@ -2923,7 +2877,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>49</v>
       </c>
@@ -2943,7 +2897,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>49</v>
       </c>
@@ -2963,7 +2917,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>49</v>
       </c>
@@ -2983,7 +2937,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>49</v>
       </c>
@@ -3003,7 +2957,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>49</v>
       </c>
@@ -3023,7 +2977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>49</v>
       </c>
@@ -3043,7 +2997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>49</v>
       </c>
@@ -3063,7 +3017,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>85</v>
       </c>
@@ -3083,7 +3037,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>85</v>
       </c>
@@ -3103,7 +3057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>85</v>
       </c>
@@ -3123,7 +3077,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>85</v>
       </c>
@@ -3143,7 +3097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>85</v>
       </c>
@@ -3163,7 +3117,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>91</v>
       </c>
@@ -3183,7 +3137,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>91</v>
       </c>
@@ -3203,7 +3157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>91</v>
       </c>
@@ -3223,7 +3177,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>91</v>
       </c>
@@ -3243,7 +3197,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>91</v>
       </c>
@@ -3263,7 +3217,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>91</v>
       </c>
@@ -3283,7 +3237,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>91</v>
       </c>
@@ -3303,7 +3257,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>91</v>
       </c>
@@ -3323,7 +3277,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>91</v>
       </c>
@@ -3343,7 +3297,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>91</v>
       </c>
@@ -3363,7 +3317,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>91</v>
       </c>
@@ -3383,7 +3337,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>91</v>
       </c>
@@ -3403,7 +3357,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>91</v>
       </c>
@@ -3423,7 +3377,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>91</v>
       </c>
@@ -3443,7 +3397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>91</v>
       </c>
@@ -3463,7 +3417,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>91</v>
       </c>
@@ -3483,7 +3437,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>91</v>
       </c>
@@ -3503,7 +3457,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>91</v>
       </c>
@@ -3523,7 +3477,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>110</v>
       </c>
@@ -3543,7 +3497,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>110</v>
       </c>
@@ -3563,7 +3517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>110</v>
       </c>
@@ -3583,7 +3537,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>110</v>
       </c>
@@ -3603,7 +3557,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>110</v>
       </c>
@@ -3623,7 +3577,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>116</v>
       </c>
@@ -3643,7 +3597,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>116</v>
       </c>
@@ -3663,7 +3617,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>116</v>
       </c>
@@ -3683,7 +3637,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>116</v>
       </c>
@@ -3703,7 +3657,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>116</v>
       </c>
@@ -3723,7 +3677,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>122</v>
       </c>
@@ -3743,7 +3697,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>122</v>
       </c>
@@ -3763,7 +3717,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>122</v>
       </c>
@@ -3783,7 +3737,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>122</v>
       </c>
@@ -3803,7 +3757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>122</v>
       </c>
@@ -3823,7 +3777,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>122</v>
       </c>
@@ -3843,7 +3797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>122</v>
       </c>
@@ -3863,7 +3817,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>122</v>
       </c>
@@ -3883,7 +3837,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>122</v>
       </c>
@@ -3903,7 +3857,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>122</v>
       </c>
@@ -3923,7 +3877,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>122</v>
       </c>
@@ -3943,7 +3897,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>122</v>
       </c>
@@ -3963,7 +3917,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>135</v>
       </c>
@@ -3983,7 +3937,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>135</v>
       </c>
@@ -4003,7 +3957,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
         <v>135</v>
       </c>
@@ -4023,7 +3977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
         <v>135</v>
       </c>
@@ -4043,7 +3997,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
         <v>135</v>
       </c>
@@ -4063,7 +4017,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>135</v>
       </c>
@@ -4083,7 +4037,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
         <v>135</v>
       </c>
@@ -4103,7 +4057,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
         <v>135</v>
       </c>
@@ -4123,7 +4077,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
         <v>135</v>
       </c>
@@ -4143,7 +4097,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>135</v>
       </c>
@@ -4163,7 +4117,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>135</v>
       </c>
@@ -4183,7 +4137,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>135</v>
       </c>
@@ -4203,7 +4157,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>135</v>
       </c>
@@ -4223,7 +4177,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>135</v>
       </c>
@@ -4243,7 +4197,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>135</v>
       </c>
@@ -4263,7 +4217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>135</v>
       </c>
@@ -4283,7 +4237,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>135</v>
       </c>
@@ -4303,7 +4257,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>135</v>
       </c>
@@ -4323,7 +4277,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>135</v>
       </c>
@@ -4343,7 +4297,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>135</v>
       </c>
@@ -4363,7 +4317,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>135</v>
       </c>
@@ -4383,7 +4337,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>135</v>
       </c>
@@ -4403,7 +4357,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>135</v>
       </c>
@@ -4423,7 +4377,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>135</v>
       </c>
@@ -4443,7 +4397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>135</v>
       </c>
@@ -4463,7 +4417,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>135</v>
       </c>
@@ -4483,7 +4437,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>135</v>
       </c>
@@ -4503,7 +4457,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>135</v>
       </c>
@@ -4523,7 +4477,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
         <v>135</v>
       </c>
@@ -4543,7 +4497,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
         <v>135</v>
       </c>
@@ -4563,7 +4517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
         <v>135</v>
       </c>
@@ -4583,7 +4537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
         <v>135</v>
       </c>
@@ -4603,7 +4557,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
         <v>135</v>
       </c>
@@ -4623,7 +4577,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
         <v>135</v>
       </c>
@@ -4643,7 +4597,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
         <v>135</v>
       </c>
@@ -4663,7 +4617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
         <v>135</v>
       </c>
@@ -4683,7 +4637,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
         <v>135</v>
       </c>
@@ -4703,7 +4657,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
         <v>135</v>
       </c>
@@ -4723,7 +4677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
         <v>135</v>
       </c>
@@ -4743,7 +4697,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>135</v>
       </c>
@@ -4763,7 +4717,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>135</v>
       </c>
@@ -4783,7 +4737,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
         <v>135</v>
       </c>
@@ -4803,7 +4757,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
         <v>135</v>
       </c>
@@ -4823,7 +4777,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="149" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
         <v>135</v>
       </c>
@@ -4843,7 +4797,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
         <v>135</v>
       </c>
@@ -4863,7 +4817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
         <v>135</v>
       </c>
@@ -4883,7 +4837,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
         <v>135</v>
       </c>
@@ -4903,7 +4857,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="153" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
         <v>135</v>
       </c>
@@ -4923,7 +4877,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
         <v>135</v>
       </c>
@@ -4943,7 +4897,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
         <v>135</v>
       </c>
@@ -4963,7 +4917,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="156" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
         <v>135</v>
       </c>
@@ -4983,7 +4937,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
         <v>135</v>
       </c>
@@ -5003,7 +4957,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="158" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
         <v>135</v>
       </c>
@@ -5023,7 +4977,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
         <v>135</v>
       </c>
@@ -5043,7 +4997,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="160" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
         <v>135</v>
       </c>
@@ -5063,7 +5017,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
         <v>135</v>
       </c>
@@ -5083,7 +5037,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
         <v>135</v>
       </c>
@@ -5103,7 +5057,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="163" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
         <v>135</v>
       </c>
@@ -5123,7 +5077,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
         <v>135</v>
       </c>
@@ -5143,7 +5097,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="165" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
         <v>195</v>
       </c>
@@ -5163,7 +5117,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
         <v>195</v>
       </c>
@@ -5183,7 +5137,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
         <v>195</v>
       </c>
@@ -5203,7 +5157,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="168" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
         <v>195</v>
       </c>
@@ -5223,7 +5177,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="169" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
         <v>200</v>
       </c>
@@ -5243,7 +5197,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="170" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
         <v>200</v>
       </c>
@@ -5263,7 +5217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="171" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
         <v>200</v>
       </c>
@@ -5283,7 +5237,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="172" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
         <v>200</v>
       </c>
@@ -5303,7 +5257,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
         <v>200</v>
       </c>
@@ -5323,7 +5277,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="174" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="27" t="s">
         <v>206</v>
       </c>
@@ -5343,7 +5297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="27" t="s">
         <v>206</v>
       </c>
@@ -5363,7 +5317,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="176" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="27" t="s">
         <v>206</v>
       </c>
@@ -5383,7 +5337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="27" t="s">
         <v>206</v>
       </c>
@@ -5403,7 +5357,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="31" t="s">
         <v>211</v>
       </c>
@@ -5423,7 +5377,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="31" t="s">
         <v>211</v>
       </c>
@@ -5443,7 +5397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="31" t="s">
         <v>211</v>
       </c>
@@ -5463,7 +5417,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="31" t="s">
         <v>211</v>
       </c>
@@ -5483,7 +5437,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="31" t="s">
         <v>211</v>
       </c>
@@ -5503,7 +5457,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="31" t="s">
         <v>211</v>
       </c>
@@ -5523,7 +5477,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="32" t="s">
         <v>218</v>
       </c>
@@ -5543,7 +5497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="32" t="s">
         <v>218</v>
       </c>
@@ -5563,7 +5517,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="32" t="s">
         <v>218</v>
       </c>
@@ -5583,7 +5537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="32" t="s">
         <v>218</v>
       </c>
@@ -5603,7 +5557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="188" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="32" t="s">
         <v>218</v>
       </c>
@@ -5623,7 +5577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="189" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="32" t="s">
         <v>218</v>
       </c>
@@ -5643,7 +5597,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="190" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="32" t="s">
         <v>218</v>
       </c>
@@ -5663,7 +5617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="191" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="32" t="s">
         <v>218</v>
       </c>
@@ -5683,7 +5637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="192" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="32" t="s">
         <v>218</v>
       </c>
@@ -5703,7 +5657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="193" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="32" t="s">
         <v>218</v>
       </c>
@@ -5723,7 +5677,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="194" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="194" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="32" t="s">
         <v>218</v>
       </c>
@@ -5743,7 +5697,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="32" t="s">
         <v>218</v>
       </c>
@@ -5763,7 +5717,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="196" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" s="32" t="s">
         <v>218</v>
       </c>
@@ -5783,7 +5737,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="197" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" s="32" t="s">
         <v>218</v>
       </c>
@@ -5803,7 +5757,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" s="32" t="s">
         <v>218</v>
       </c>
@@ -5823,7 +5777,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="199" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" s="32" t="s">
         <v>218</v>
       </c>
@@ -5843,7 +5797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" s="33" t="s">
         <v>235</v>
       </c>
@@ -5863,7 +5817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="201" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="201" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" s="33" t="s">
         <v>235</v>
       </c>
@@ -5883,7 +5837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="202" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="202" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" s="33" t="s">
         <v>235</v>
       </c>
@@ -5903,7 +5857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="203" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" s="33" t="s">
         <v>235</v>
       </c>
@@ -5923,7 +5877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="204" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" s="33" t="s">
         <v>235</v>
       </c>
@@ -5943,7 +5897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="205" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="33" t="s">
         <v>235</v>
       </c>
@@ -5963,7 +5917,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="206" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" s="33" t="s">
         <v>235</v>
       </c>
@@ -5983,7 +5937,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="207" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" s="33" t="s">
         <v>235</v>
       </c>
@@ -6003,7 +5957,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="208" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" s="33" t="s">
         <v>235</v>
       </c>
@@ -6023,7 +5977,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="209" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="33" t="s">
         <v>235</v>
       </c>
@@ -6043,11 +5997,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A210" s="34" t="s">
+    <row r="210" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B210" s="35" t="s">
+      <c r="B210" s="28" t="s">
         <v>246</v>
       </c>
       <c r="C210" s="29">
@@ -6056,18 +6010,18 @@
       <c r="D210" s="30">
         <v>5000</v>
       </c>
-      <c r="E210" s="36">
+      <c r="E210" s="15">
         <v>5000</v>
       </c>
-      <c r="F210" s="37" t="s">
+      <c r="F210" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A211" s="34" t="s">
+    <row r="211" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A211" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B211" s="35" t="s">
+      <c r="B211" s="28" t="s">
         <v>247</v>
       </c>
       <c r="C211" s="29">
@@ -6076,18 +6030,18 @@
       <c r="D211" s="30">
         <v>5000</v>
       </c>
-      <c r="E211" s="36">
+      <c r="E211" s="15">
         <v>5000</v>
       </c>
-      <c r="F211" s="37" t="s">
+      <c r="F211" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A212" s="34" t="s">
+    <row r="212" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B212" s="35" t="s">
+      <c r="B212" s="28" t="s">
         <v>248</v>
       </c>
       <c r="C212" s="29">
@@ -6096,18 +6050,18 @@
       <c r="D212" s="30">
         <v>5000</v>
       </c>
-      <c r="E212" s="36">
+      <c r="E212" s="15">
         <v>5000</v>
       </c>
-      <c r="F212" s="37" t="s">
+      <c r="F212" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A213" s="34" t="s">
+    <row r="213" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A213" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B213" s="35" t="s">
+      <c r="B213" s="28" t="s">
         <v>249</v>
       </c>
       <c r="C213" s="29">
@@ -6116,18 +6070,18 @@
       <c r="D213" s="30">
         <v>5000</v>
       </c>
-      <c r="E213" s="36">
+      <c r="E213" s="15">
         <v>5000</v>
       </c>
-      <c r="F213" s="37" t="s">
+      <c r="F213" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A214" s="34" t="s">
+    <row r="214" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A214" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B214" s="35" t="s">
+      <c r="B214" s="28" t="s">
         <v>250</v>
       </c>
       <c r="C214" s="29">
@@ -6136,18 +6090,18 @@
       <c r="D214" s="30">
         <v>5000</v>
       </c>
-      <c r="E214" s="36">
+      <c r="E214" s="15">
         <v>5000</v>
       </c>
-      <c r="F214" s="37" t="s">
+      <c r="F214" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A215" s="34" t="s">
+    <row r="215" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A215" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B215" s="35" t="s">
+      <c r="B215" s="28" t="s">
         <v>251</v>
       </c>
       <c r="C215" s="29">
@@ -6156,18 +6110,18 @@
       <c r="D215" s="30">
         <v>5000</v>
       </c>
-      <c r="E215" s="36">
+      <c r="E215" s="15">
         <v>5000</v>
       </c>
-      <c r="F215" s="37" t="s">
+      <c r="F215" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A216" s="34" t="s">
+    <row r="216" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B216" s="35" t="s">
+      <c r="B216" s="28" t="s">
         <v>252</v>
       </c>
       <c r="C216" s="29">
@@ -6176,18 +6130,18 @@
       <c r="D216" s="30">
         <v>10000</v>
       </c>
-      <c r="E216" s="36">
-        <v>10000</v>
-      </c>
-      <c r="F216" s="37" t="s">
+      <c r="E216" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F216" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A217" s="34" t="s">
+    <row r="217" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A217" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B217" s="35" t="s">
+      <c r="B217" s="28" t="s">
         <v>253</v>
       </c>
       <c r="C217" s="29">
@@ -6196,18 +6150,18 @@
       <c r="D217" s="30">
         <v>15000</v>
       </c>
-      <c r="E217" s="36">
+      <c r="E217" s="15">
         <v>15000</v>
       </c>
-      <c r="F217" s="37" t="s">
+      <c r="F217" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A218" s="34" t="s">
+    <row r="218" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A218" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B218" s="35" t="s">
+      <c r="B218" s="28" t="s">
         <v>254</v>
       </c>
       <c r="C218" s="29">
@@ -6216,18 +6170,18 @@
       <c r="D218" s="30">
         <v>15000</v>
       </c>
-      <c r="E218" s="36">
+      <c r="E218" s="15">
         <v>15000</v>
       </c>
-      <c r="F218" s="37" t="s">
+      <c r="F218" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A219" s="34" t="s">
+    <row r="219" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A219" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B219" s="35" t="s">
+      <c r="B219" s="28" t="s">
         <v>255</v>
       </c>
       <c r="C219" s="29">
@@ -6236,18 +6190,18 @@
       <c r="D219" s="30">
         <v>15000</v>
       </c>
-      <c r="E219" s="36">
+      <c r="E219" s="15">
         <v>15000</v>
       </c>
-      <c r="F219" s="37" t="s">
+      <c r="F219" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="220" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A220" s="34" t="s">
+    <row r="220" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A220" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B220" s="35" t="s">
+      <c r="B220" s="28" t="s">
         <v>256</v>
       </c>
       <c r="C220" s="29">
@@ -6256,18 +6210,18 @@
       <c r="D220" s="30">
         <v>15000</v>
       </c>
-      <c r="E220" s="36">
+      <c r="E220" s="15">
         <v>15000</v>
       </c>
-      <c r="F220" s="37" t="s">
+      <c r="F220" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="221" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A221" s="34" t="s">
+    <row r="221" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A221" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B221" s="35" t="s">
+      <c r="B221" s="28" t="s">
         <v>257</v>
       </c>
       <c r="C221" s="29">
@@ -6276,18 +6230,18 @@
       <c r="D221" s="30">
         <v>15000</v>
       </c>
-      <c r="E221" s="36">
+      <c r="E221" s="15">
         <v>15000</v>
       </c>
-      <c r="F221" s="37" t="s">
+      <c r="F221" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="222" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A222" s="34" t="s">
+    <row r="222" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A222" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B222" s="35" t="s">
+      <c r="B222" s="28" t="s">
         <v>258</v>
       </c>
       <c r="C222" s="29">
@@ -6296,18 +6250,18 @@
       <c r="D222" s="30">
         <v>15000</v>
       </c>
-      <c r="E222" s="36">
+      <c r="E222" s="15">
         <v>15000</v>
       </c>
-      <c r="F222" s="37" t="s">
+      <c r="F222" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A223" s="38" t="s">
+    <row r="223" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A223" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B223" s="39" t="s">
+      <c r="B223" s="20" t="s">
         <v>259</v>
       </c>
       <c r="C223" s="21">
@@ -6316,18 +6270,18 @@
       <c r="D223" s="22">
         <v>5000</v>
       </c>
-      <c r="E223" s="36">
+      <c r="E223" s="15">
         <v>5000</v>
       </c>
-      <c r="F223" s="37" t="s">
+      <c r="F223" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A224" s="38" t="s">
+    <row r="224" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A224" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B224" s="39" t="s">
+      <c r="B224" s="20" t="s">
         <v>260</v>
       </c>
       <c r="C224" s="21">
@@ -6336,18 +6290,18 @@
       <c r="D224" s="22">
         <v>8000</v>
       </c>
-      <c r="E224" s="36">
+      <c r="E224" s="15">
         <v>8000</v>
       </c>
-      <c r="F224" s="37" t="s">
+      <c r="F224" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="225" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A225" s="38" t="s">
+    <row r="225" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A225" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B225" s="39" t="s">
+      <c r="B225" s="20" t="s">
         <v>261</v>
       </c>
       <c r="C225" s="21">
@@ -6356,18 +6310,18 @@
       <c r="D225" s="22">
         <v>8000</v>
       </c>
-      <c r="E225" s="36">
+      <c r="E225" s="15">
         <v>8000</v>
       </c>
-      <c r="F225" s="37" t="s">
+      <c r="F225" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A226" s="38" t="s">
+    <row r="226" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A226" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B226" s="39" t="s">
+      <c r="B226" s="20" t="s">
         <v>262</v>
       </c>
       <c r="C226" s="21">
@@ -6376,18 +6330,18 @@
       <c r="D226" s="22">
         <v>8000</v>
       </c>
-      <c r="E226" s="36">
+      <c r="E226" s="15">
         <v>8000</v>
       </c>
-      <c r="F226" s="37" t="s">
+      <c r="F226" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="227" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A227" s="38" t="s">
+    <row r="227" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A227" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B227" s="39" t="s">
+      <c r="B227" s="20" t="s">
         <v>263</v>
       </c>
       <c r="C227" s="21">
@@ -6396,18 +6350,18 @@
       <c r="D227" s="22">
         <v>5000</v>
       </c>
-      <c r="E227" s="36">
+      <c r="E227" s="15">
         <v>5000</v>
       </c>
-      <c r="F227" s="37" t="s">
+      <c r="F227" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="228" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A228" s="38" t="s">
+    <row r="228" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A228" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B228" s="39" t="s">
+      <c r="B228" s="20" t="s">
         <v>264</v>
       </c>
       <c r="C228" s="21">
@@ -6416,18 +6370,18 @@
       <c r="D228" s="22">
         <v>10000</v>
       </c>
-      <c r="E228" s="36">
-        <v>10000</v>
-      </c>
-      <c r="F228" s="37" t="s">
+      <c r="E228" s="15">
+        <v>10000</v>
+      </c>
+      <c r="F228" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="229" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A229" s="38" t="s">
+    <row r="229" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A229" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B229" s="39" t="s">
+      <c r="B229" s="20" t="s">
         <v>265</v>
       </c>
       <c r="C229" s="21">
@@ -6436,18 +6390,18 @@
       <c r="D229" s="22">
         <v>8000</v>
       </c>
-      <c r="E229" s="36">
+      <c r="E229" s="15">
         <v>8000</v>
       </c>
-      <c r="F229" s="37" t="s">
+      <c r="F229" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="230" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A230" s="38" t="s">
+    <row r="230" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A230" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="B230" s="39" t="s">
+      <c r="B230" s="20" t="s">
         <v>266</v>
       </c>
       <c r="C230" s="21">
@@ -6456,18 +6410,18 @@
       <c r="D230" s="22">
         <v>15000</v>
       </c>
-      <c r="E230" s="36">
+      <c r="E230" s="15">
         <v>15000</v>
       </c>
-      <c r="F230" s="37" t="s">
+      <c r="F230" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="231" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A231" s="40" t="s">
+    <row r="231" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A231" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B231" s="35" t="s">
+      <c r="B231" s="28" t="s">
         <v>268</v>
       </c>
       <c r="C231" s="29">
@@ -6476,18 +6430,18 @@
       <c r="D231" s="30">
         <v>3500</v>
       </c>
-      <c r="E231" s="36">
+      <c r="E231" s="15">
         <v>3500</v>
       </c>
-      <c r="F231" s="37" t="s">
+      <c r="F231" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="232" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A232" s="40" t="s">
+    <row r="232" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A232" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B232" s="35" t="s">
+      <c r="B232" s="28" t="s">
         <v>269</v>
       </c>
       <c r="C232" s="29">
@@ -6496,18 +6450,18 @@
       <c r="D232" s="30">
         <v>3500</v>
       </c>
-      <c r="E232" s="36">
+      <c r="E232" s="15">
         <v>3500</v>
       </c>
-      <c r="F232" s="37" t="s">
+      <c r="F232" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="233" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A233" s="40" t="s">
+    <row r="233" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A233" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B233" s="35" t="s">
+      <c r="B233" s="28" t="s">
         <v>270</v>
       </c>
       <c r="C233" s="29">
@@ -6516,18 +6470,18 @@
       <c r="D233" s="30">
         <v>3500</v>
       </c>
-      <c r="E233" s="36">
+      <c r="E233" s="15">
         <v>3500</v>
       </c>
-      <c r="F233" s="37" t="s">
+      <c r="F233" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A234" s="40" t="s">
+    <row r="234" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A234" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B234" s="35" t="s">
+      <c r="B234" s="28" t="s">
         <v>271</v>
       </c>
       <c r="C234" s="29">
@@ -6536,18 +6490,18 @@
       <c r="D234" s="30">
         <v>3500</v>
       </c>
-      <c r="E234" s="36">
+      <c r="E234" s="15">
         <v>3500</v>
       </c>
-      <c r="F234" s="37" t="s">
+      <c r="F234" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="235" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A235" s="40" t="s">
+    <row r="235" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B235" s="35" t="s">
+      <c r="B235" s="28" t="s">
         <v>272</v>
       </c>
       <c r="C235" s="29">
@@ -6556,18 +6510,18 @@
       <c r="D235" s="30">
         <v>3500</v>
       </c>
-      <c r="E235" s="36">
+      <c r="E235" s="15">
         <v>3500</v>
       </c>
-      <c r="F235" s="37" t="s">
+      <c r="F235" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="236" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A236" s="40" t="s">
+    <row r="236" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B236" s="35" t="s">
+      <c r="B236" s="28" t="s">
         <v>273</v>
       </c>
       <c r="C236" s="29">
@@ -6576,18 +6530,18 @@
       <c r="D236" s="30">
         <v>3500</v>
       </c>
-      <c r="E236" s="36">
+      <c r="E236" s="15">
         <v>3500</v>
       </c>
-      <c r="F236" s="37" t="s">
+      <c r="F236" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="237" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A237" s="40" t="s">
+    <row r="237" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B237" s="35" t="s">
+      <c r="B237" s="28" t="s">
         <v>274</v>
       </c>
       <c r="C237" s="29">
@@ -6596,18 +6550,18 @@
       <c r="D237" s="30">
         <v>3500</v>
       </c>
-      <c r="E237" s="36">
+      <c r="E237" s="15">
         <v>3500</v>
       </c>
-      <c r="F237" s="37" t="s">
+      <c r="F237" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A238" s="40" t="s">
+    <row r="238" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B238" s="35" t="s">
+      <c r="B238" s="28" t="s">
         <v>275</v>
       </c>
       <c r="C238" s="29">
@@ -6616,18 +6570,18 @@
       <c r="D238" s="30">
         <v>3500</v>
       </c>
-      <c r="E238" s="36">
+      <c r="E238" s="15">
         <v>3500</v>
       </c>
-      <c r="F238" s="37" t="s">
+      <c r="F238" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="239" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A239" s="40" t="s">
+    <row r="239" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B239" s="35" t="s">
+      <c r="B239" s="28" t="s">
         <v>276</v>
       </c>
       <c r="C239" s="29">
@@ -6636,18 +6590,18 @@
       <c r="D239" s="30">
         <v>3500</v>
       </c>
-      <c r="E239" s="36">
+      <c r="E239" s="15">
         <v>3500</v>
       </c>
-      <c r="F239" s="37" t="s">
+      <c r="F239" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="240" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A240" s="40" t="s">
+    <row r="240" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B240" s="35" t="s">
+      <c r="B240" s="28" t="s">
         <v>277</v>
       </c>
       <c r="C240" s="29">
@@ -6656,18 +6610,18 @@
       <c r="D240" s="30">
         <v>3500</v>
       </c>
-      <c r="E240" s="36">
+      <c r="E240" s="15">
         <v>3500</v>
       </c>
-      <c r="F240" s="37" t="s">
+      <c r="F240" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A241" s="40" t="s">
+    <row r="241" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A241" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B241" s="35" t="s">
+      <c r="B241" s="28" t="s">
         <v>278</v>
       </c>
       <c r="C241" s="29">
@@ -6676,18 +6630,18 @@
       <c r="D241" s="30">
         <v>3500</v>
       </c>
-      <c r="E241" s="36">
+      <c r="E241" s="15">
         <v>3500</v>
       </c>
-      <c r="F241" s="37" t="s">
+      <c r="F241" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A242" s="40" t="s">
+    <row r="242" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A242" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B242" s="35" t="s">
+      <c r="B242" s="28" t="s">
         <v>279</v>
       </c>
       <c r="C242" s="29">
@@ -6696,18 +6650,18 @@
       <c r="D242" s="30">
         <v>3500</v>
       </c>
-      <c r="E242" s="36">
+      <c r="E242" s="15">
         <v>3500</v>
       </c>
-      <c r="F242" s="37" t="s">
+      <c r="F242" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="243" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A243" s="40" t="s">
+    <row r="243" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A243" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B243" s="35" t="s">
+      <c r="B243" s="28" t="s">
         <v>280</v>
       </c>
       <c r="C243" s="29">
@@ -6716,18 +6670,18 @@
       <c r="D243" s="30">
         <v>3500</v>
       </c>
-      <c r="E243" s="36">
+      <c r="E243" s="15">
         <v>3500</v>
       </c>
-      <c r="F243" s="37" t="s">
+      <c r="F243" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A244" s="40" t="s">
+    <row r="244" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A244" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B244" s="35" t="s">
+      <c r="B244" s="28" t="s">
         <v>281</v>
       </c>
       <c r="C244" s="29">
@@ -6736,18 +6690,18 @@
       <c r="D244" s="30">
         <v>3500</v>
       </c>
-      <c r="E244" s="36">
+      <c r="E244" s="15">
         <v>3500</v>
       </c>
-      <c r="F244" s="37" t="s">
+      <c r="F244" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="245" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A245" s="40" t="s">
+    <row r="245" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A245" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B245" s="35" t="s">
+      <c r="B245" s="28" t="s">
         <v>282</v>
       </c>
       <c r="C245" s="29">
@@ -6756,18 +6710,18 @@
       <c r="D245" s="30">
         <v>3500</v>
       </c>
-      <c r="E245" s="36">
+      <c r="E245" s="15">
         <v>3500</v>
       </c>
-      <c r="F245" s="37" t="s">
+      <c r="F245" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A246" s="40" t="s">
+    <row r="246" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A246" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="B246" s="35" t="s">
+      <c r="B246" s="28" t="s">
         <v>283</v>
       </c>
       <c r="C246" s="29">
@@ -6776,24 +6730,24 @@
       <c r="D246" s="30">
         <v>3500</v>
       </c>
-      <c r="E246" s="36">
+      <c r="E246" s="15">
         <v>3500</v>
       </c>
-      <c r="F246" s="37" t="s">
+      <c r="F246" s="26" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F246" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:F246"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -6802,263 +6756,263 @@
     <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="35" t="s">
         <v>284</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="C1" s="35" t="s">
         <v>285</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="35" t="s">
         <v>286</v>
       </c>
-      <c r="E1" s="41" t="s">
+      <c r="E1" s="35" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+    <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="43">
+      <c r="B2" s="37">
         <v>24</v>
       </c>
-      <c r="C2" s="44">
+      <c r="C2" s="38">
         <v>4.93</v>
       </c>
-      <c r="D2" s="45">
+      <c r="D2" s="39">
         <v>4200</v>
       </c>
-      <c r="E2" s="45">
+      <c r="E2" s="39">
         <v>7208</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="47">
+      <c r="B3" s="41">
         <v>35</v>
       </c>
-      <c r="C3" s="48">
+      <c r="C3" s="42">
         <v>7.46</v>
       </c>
-      <c r="D3" s="49">
+      <c r="D3" s="43">
         <v>6857</v>
       </c>
-      <c r="E3" s="49">
+      <c r="E3" s="43">
         <v>11186</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="50" t="s">
+    <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="51">
+      <c r="B4" s="45">
         <v>5</v>
       </c>
-      <c r="C4" s="52">
+      <c r="C4" s="46">
         <v>11.5</v>
       </c>
-      <c r="D4" s="53">
+      <c r="D4" s="47">
         <v>7400</v>
       </c>
-      <c r="E4" s="53">
+      <c r="E4" s="47">
         <v>17200</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="54" t="s">
+    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="55">
+      <c r="B5" s="49">
         <v>18</v>
       </c>
-      <c r="C5" s="56">
+      <c r="C5" s="50">
         <v>6.47</v>
       </c>
-      <c r="D5" s="57">
+      <c r="D5" s="51">
         <v>6639</v>
       </c>
-      <c r="E5" s="57">
+      <c r="E5" s="51">
         <v>9556</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="B6" s="59">
+      <c r="B6" s="53">
         <v>5</v>
       </c>
-      <c r="C6" s="60">
+      <c r="C6" s="54">
         <v>8</v>
       </c>
-      <c r="D6" s="61">
+      <c r="D6" s="55">
         <v>6000</v>
       </c>
-      <c r="E6" s="61">
+      <c r="E6" s="55">
         <v>12000</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="62" t="s">
+    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="56" t="s">
         <v>116</v>
       </c>
-      <c r="B7" s="63">
+      <c r="B7" s="57">
         <v>5</v>
       </c>
-      <c r="C7" s="64">
+      <c r="C7" s="58">
         <v>11.18</v>
       </c>
-      <c r="D7" s="65">
+      <c r="D7" s="59">
         <v>4600</v>
       </c>
-      <c r="E7" s="65">
+      <c r="E7" s="59">
         <v>16800</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="66" t="s">
+    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="60" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="67">
+      <c r="B8" s="61">
         <v>12</v>
       </c>
-      <c r="C8" s="68">
+      <c r="C8" s="62">
         <v>16.25</v>
       </c>
-      <c r="D8" s="69">
+      <c r="D8" s="63">
         <v>8167</v>
       </c>
-      <c r="E8" s="69">
+      <c r="E8" s="63">
         <v>24375</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="s">
+    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="B9" s="71">
+      <c r="B9" s="65">
         <v>59</v>
       </c>
-      <c r="C9" s="72">
+      <c r="C9" s="66">
         <v>25.85</v>
       </c>
-      <c r="D9" s="73">
+      <c r="D9" s="67">
         <v>7051</v>
       </c>
-      <c r="E9" s="73">
+      <c r="E9" s="67">
         <v>38771</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="74" t="s">
+    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="68" t="s">
         <v>195</v>
       </c>
-      <c r="B10" s="75">
+      <c r="B10" s="69">
         <v>4</v>
       </c>
-      <c r="C10" s="76">
+      <c r="C10" s="70">
         <v>28</v>
       </c>
-      <c r="D10" s="77">
+      <c r="D10" s="71">
         <v>10750</v>
       </c>
-      <c r="E10" s="77">
+      <c r="E10" s="71">
         <v>42000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="78" t="s">
+    <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="72" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="79">
+      <c r="B11" s="73">
         <v>5</v>
       </c>
-      <c r="C11" s="80">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="D11" s="81">
+      <c r="C11" s="74">
+        <v>10.2</v>
+      </c>
+      <c r="D11" s="75">
         <v>2000</v>
       </c>
-      <c r="E11" s="81">
+      <c r="E11" s="75">
         <v>15300</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="66" t="s">
+    <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="60" t="s">
         <v>206</v>
       </c>
-      <c r="B12" s="67">
+      <c r="B12" s="61">
         <v>4</v>
       </c>
-      <c r="C12" s="68">
+      <c r="C12" s="62">
         <v>4.63</v>
       </c>
-      <c r="D12" s="69">
+      <c r="D12" s="63">
         <v>2750</v>
       </c>
-      <c r="E12" s="69">
+      <c r="E12" s="63">
         <v>2750</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62" t="s">
+    <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="56" t="s">
         <v>211</v>
       </c>
-      <c r="B13" s="63">
+      <c r="B13" s="57">
         <v>6</v>
       </c>
-      <c r="C13" s="64">
+      <c r="C13" s="58">
         <v>3.33</v>
       </c>
-      <c r="D13" s="65">
+      <c r="D13" s="59">
         <v>2317</v>
       </c>
-      <c r="E13" s="65">
+      <c r="E13" s="59">
         <v>2317</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="82" t="s">
+    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="76" t="s">
         <v>218</v>
       </c>
-      <c r="B14" s="83">
+      <c r="B14" s="77">
         <v>16</v>
       </c>
-      <c r="C14" s="84">
+      <c r="C14" s="78">
         <v>10.19</v>
       </c>
-      <c r="D14" s="85">
+      <c r="D14" s="79">
         <v>7563</v>
       </c>
-      <c r="E14" s="85">
+      <c r="E14" s="79">
         <v>7563</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="70" t="s">
+    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="64" t="s">
         <v>235</v>
       </c>
-      <c r="B15" s="71">
-        <v>10</v>
-      </c>
-      <c r="C15" s="72">
+      <c r="B15" s="65">
+        <v>10</v>
+      </c>
+      <c r="C15" s="66">
         <v>11.6</v>
       </c>
-      <c r="D15" s="73">
+      <c r="D15" s="67">
         <v>9650</v>
       </c>
-      <c r="E15" s="73">
+      <c r="E15" s="67">
         <v>9650</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update spreadsheets and products-list after new product additions
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis.xlsx
+++ b/AmericanSelect_PricingAnalysis.xlsx
@@ -1,20 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53709643-D209-4CF4-B55A-984AFBEF98D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Legend" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Pricing Analysis" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Summary by Category" state="visible" r:id="rId6"/>
+    <sheet name="Legend" sheetId="1" r:id="rId1"/>
+    <sheet name="Pricing Analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary by Category" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pricing Analysis'!$A$1:$F$246</definedName>
     <definedName name="_xlnm._FilterDatabase">'Pricing Analysis'!$A$1:$F$173</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -888,39 +895,39 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0 &quot;XAF&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0\ &quot;XAF&quot;"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="10"/>
       <color rgb="FF1A237E"/>
-      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -934,20 +941,20 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
-      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF4A0070"/>
-      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1719,15 +1726,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1735,7 +1742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1743,7 +1750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1751,7 +1758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1759,7 +1766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -1767,7 +1774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1775,7 +1782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -1783,7 +1790,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
@@ -1791,7 +1798,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
@@ -1801,14 +1808,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F246"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="58" customWidth="1"/>
@@ -1817,7 +1825,7 @@
     <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>18</v>
       </c>
@@ -1837,7 +1845,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>24</v>
       </c>
@@ -1857,7 +1865,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>24</v>
       </c>
@@ -1877,7 +1885,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>24</v>
       </c>
@@ -1897,7 +1905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
@@ -1917,7 +1925,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>24</v>
       </c>
@@ -1937,7 +1945,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>24</v>
       </c>
@@ -1957,7 +1965,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>24</v>
       </c>
@@ -1977,7 +1985,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>24</v>
       </c>
@@ -1997,7 +2005,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>24</v>
       </c>
@@ -2017,7 +2025,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>24</v>
       </c>
@@ -2037,7 +2045,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>24</v>
       </c>
@@ -2057,7 +2065,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>24</v>
       </c>
@@ -2077,7 +2085,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>24</v>
       </c>
@@ -2097,7 +2105,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>24</v>
       </c>
@@ -2117,7 +2125,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
@@ -2137,7 +2145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>24</v>
       </c>
@@ -2157,7 +2165,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>24</v>
       </c>
@@ -2177,7 +2185,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>24</v>
       </c>
@@ -2197,7 +2205,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>24</v>
       </c>
@@ -2217,7 +2225,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>24</v>
       </c>
@@ -2237,7 +2245,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>24</v>
       </c>
@@ -2257,7 +2265,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>24</v>
       </c>
@@ -2277,7 +2285,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>24</v>
       </c>
@@ -2297,7 +2305,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>24</v>
       </c>
@@ -2317,7 +2325,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>49</v>
       </c>
@@ -2337,7 +2345,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>49</v>
       </c>
@@ -2357,7 +2365,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>49</v>
       </c>
@@ -2377,7 +2385,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>49</v>
       </c>
@@ -2397,7 +2405,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>49</v>
       </c>
@@ -2417,7 +2425,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>49</v>
       </c>
@@ -2437,7 +2445,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>49</v>
       </c>
@@ -2457,7 +2465,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>49</v>
       </c>
@@ -2477,7 +2485,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>49</v>
       </c>
@@ -2497,7 +2505,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>49</v>
       </c>
@@ -2517,7 +2525,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>49</v>
       </c>
@@ -2537,7 +2545,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>49</v>
       </c>
@@ -2557,7 +2565,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>49</v>
       </c>
@@ -2577,7 +2585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>49</v>
       </c>
@@ -2597,7 +2605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>49</v>
       </c>
@@ -2617,7 +2625,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>49</v>
       </c>
@@ -2637,7 +2645,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>49</v>
       </c>
@@ -2657,7 +2665,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>49</v>
       </c>
@@ -2677,7 +2685,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>49</v>
       </c>
@@ -2697,7 +2705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>49</v>
       </c>
@@ -2717,7 +2725,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>49</v>
       </c>
@@ -2737,7 +2745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>49</v>
       </c>
@@ -2757,7 +2765,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>49</v>
       </c>
@@ -2777,7 +2785,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>49</v>
       </c>
@@ -2797,7 +2805,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>49</v>
       </c>
@@ -2817,7 +2825,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>49</v>
       </c>
@@ -2837,7 +2845,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>49</v>
       </c>
@@ -2857,7 +2865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>49</v>
       </c>
@@ -2877,7 +2885,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>49</v>
       </c>
@@ -2897,7 +2905,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>49</v>
       </c>
@@ -2917,7 +2925,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>49</v>
       </c>
@@ -2937,7 +2945,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>49</v>
       </c>
@@ -2957,7 +2965,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>49</v>
       </c>
@@ -2977,7 +2985,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>49</v>
       </c>
@@ -2997,7 +3005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>49</v>
       </c>
@@ -3017,7 +3025,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>85</v>
       </c>
@@ -3037,7 +3045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>85</v>
       </c>
@@ -3057,7 +3065,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>85</v>
       </c>
@@ -3077,7 +3085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>85</v>
       </c>
@@ -3097,7 +3105,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>85</v>
       </c>
@@ -3117,7 +3125,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>91</v>
       </c>
@@ -3137,7 +3145,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>91</v>
       </c>
@@ -3157,7 +3165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>91</v>
       </c>
@@ -3177,7 +3185,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>91</v>
       </c>
@@ -3197,7 +3205,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>91</v>
       </c>
@@ -3217,7 +3225,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>91</v>
       </c>
@@ -3237,7 +3245,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>91</v>
       </c>
@@ -3257,7 +3265,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>91</v>
       </c>
@@ -3277,7 +3285,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>91</v>
       </c>
@@ -3297,7 +3305,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>91</v>
       </c>
@@ -3317,7 +3325,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>91</v>
       </c>
@@ -3337,7 +3345,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>91</v>
       </c>
@@ -3357,7 +3365,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>91</v>
       </c>
@@ -3377,7 +3385,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>91</v>
       </c>
@@ -3397,7 +3405,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>91</v>
       </c>
@@ -3417,7 +3425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>91</v>
       </c>
@@ -3437,7 +3445,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>91</v>
       </c>
@@ -3457,7 +3465,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>91</v>
       </c>
@@ -3477,7 +3485,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>110</v>
       </c>
@@ -3497,7 +3505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>110</v>
       </c>
@@ -3517,7 +3525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>110</v>
       </c>
@@ -3537,7 +3545,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>110</v>
       </c>
@@ -3557,7 +3565,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>110</v>
       </c>
@@ -3577,7 +3585,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>116</v>
       </c>
@@ -3597,7 +3605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>116</v>
       </c>
@@ -3617,7 +3625,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>116</v>
       </c>
@@ -3637,7 +3645,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>116</v>
       </c>
@@ -3657,7 +3665,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>116</v>
       </c>
@@ -3677,7 +3685,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>122</v>
       </c>
@@ -3697,7 +3705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>122</v>
       </c>
@@ -3717,7 +3725,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>122</v>
       </c>
@@ -3737,7 +3745,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>122</v>
       </c>
@@ -3757,7 +3765,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>122</v>
       </c>
@@ -3777,7 +3785,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="99" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>122</v>
       </c>
@@ -3797,7 +3805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="100" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>122</v>
       </c>
@@ -3817,7 +3825,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>122</v>
       </c>
@@ -3837,7 +3845,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="102" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>122</v>
       </c>
@@ -3857,7 +3865,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>122</v>
       </c>
@@ -3877,7 +3885,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>122</v>
       </c>
@@ -3897,7 +3905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>122</v>
       </c>
@@ -3917,7 +3925,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>135</v>
       </c>
@@ -3937,7 +3945,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>135</v>
       </c>
@@ -3957,7 +3965,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
         <v>135</v>
       </c>
@@ -3977,7 +3985,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
         <v>135</v>
       </c>
@@ -3997,7 +4005,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="110" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
         <v>135</v>
       </c>
@@ -4017,7 +4025,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>135</v>
       </c>
@@ -4037,7 +4045,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
         <v>135</v>
       </c>
@@ -4057,7 +4065,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
         <v>135</v>
       </c>
@@ -4077,7 +4085,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="114" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
         <v>135</v>
       </c>
@@ -4097,7 +4105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>135</v>
       </c>
@@ -4117,7 +4125,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>135</v>
       </c>
@@ -4137,7 +4145,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>135</v>
       </c>
@@ -4157,7 +4165,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>135</v>
       </c>
@@ -4177,7 +4185,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="119" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>135</v>
       </c>
@@ -4197,7 +4205,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>135</v>
       </c>
@@ -4217,7 +4225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>135</v>
       </c>
@@ -4237,7 +4245,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>135</v>
       </c>
@@ -4257,7 +4265,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="123" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>135</v>
       </c>
@@ -4277,7 +4285,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>135</v>
       </c>
@@ -4297,7 +4305,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>135</v>
       </c>
@@ -4317,7 +4325,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>135</v>
       </c>
@@ -4337,7 +4345,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>135</v>
       </c>
@@ -4357,7 +4365,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="128" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>135</v>
       </c>
@@ -4377,7 +4385,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="129" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>135</v>
       </c>
@@ -4397,7 +4405,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>135</v>
       </c>
@@ -4417,7 +4425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>135</v>
       </c>
@@ -4437,7 +4445,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>135</v>
       </c>
@@ -4457,7 +4465,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>135</v>
       </c>
@@ -4477,7 +4485,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
         <v>135</v>
       </c>
@@ -4497,7 +4505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
         <v>135</v>
       </c>
@@ -4517,7 +4525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
         <v>135</v>
       </c>
@@ -4537,7 +4545,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
         <v>135</v>
       </c>
@@ -4557,7 +4565,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
         <v>135</v>
       </c>
@@ -4577,7 +4585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
         <v>135</v>
       </c>
@@ -4597,7 +4605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
         <v>135</v>
       </c>
@@ -4617,7 +4625,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
         <v>135</v>
       </c>
@@ -4637,7 +4645,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
         <v>135</v>
       </c>
@@ -4657,7 +4665,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
         <v>135</v>
       </c>
@@ -4677,7 +4685,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="144" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
         <v>135</v>
       </c>
@@ -4697,7 +4705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="145" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>135</v>
       </c>
@@ -4717,7 +4725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>135</v>
       </c>
@@ -4737,7 +4745,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="147" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
         <v>135</v>
       </c>
@@ -4757,7 +4765,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="148" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
         <v>135</v>
       </c>
@@ -4777,7 +4785,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="149" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
         <v>135</v>
       </c>
@@ -4797,7 +4805,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
         <v>135</v>
       </c>
@@ -4817,7 +4825,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
         <v>135</v>
       </c>
@@ -4837,7 +4845,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
         <v>135</v>
       </c>
@@ -4857,7 +4865,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="153" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
         <v>135</v>
       </c>
@@ -4877,7 +4885,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
         <v>135</v>
       </c>
@@ -4897,7 +4905,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
         <v>135</v>
       </c>
@@ -4917,7 +4925,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="156" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
         <v>135</v>
       </c>
@@ -4937,7 +4945,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
         <v>135</v>
       </c>
@@ -4957,7 +4965,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="158" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
         <v>135</v>
       </c>
@@ -4977,7 +4985,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
         <v>135</v>
       </c>
@@ -4997,7 +5005,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="160" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
         <v>135</v>
       </c>
@@ -5017,7 +5025,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
         <v>135</v>
       </c>
@@ -5037,7 +5045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
         <v>135</v>
       </c>
@@ -5057,7 +5065,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="163" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
         <v>135</v>
       </c>
@@ -5077,7 +5085,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
         <v>135</v>
       </c>
@@ -5097,7 +5105,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="165" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
         <v>195</v>
       </c>
@@ -5117,7 +5125,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
         <v>195</v>
       </c>
@@ -5137,7 +5145,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="167" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
         <v>195</v>
       </c>
@@ -5157,7 +5165,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="168" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
         <v>195</v>
       </c>
@@ -5177,7 +5185,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="169" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
         <v>200</v>
       </c>
@@ -5197,7 +5205,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="170" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
         <v>200</v>
       </c>
@@ -5217,7 +5225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="171" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
         <v>200</v>
       </c>
@@ -5237,7 +5245,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="172" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
         <v>200</v>
       </c>
@@ -5257,7 +5265,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="173" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
         <v>200</v>
       </c>
@@ -5277,7 +5285,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="174" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="27" t="s">
         <v>206</v>
       </c>
@@ -5297,7 +5305,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="27" t="s">
         <v>206</v>
       </c>
@@ -5317,7 +5325,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="176" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="27" t="s">
         <v>206</v>
       </c>
@@ -5337,7 +5345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="177" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="27" t="s">
         <v>206</v>
       </c>
@@ -5357,7 +5365,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="31" t="s">
         <v>211</v>
       </c>
@@ -5377,7 +5385,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="179" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="31" t="s">
         <v>211</v>
       </c>
@@ -5397,7 +5405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="31" t="s">
         <v>211</v>
       </c>
@@ -5417,7 +5425,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="181" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="31" t="s">
         <v>211</v>
       </c>
@@ -5437,7 +5445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="182" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="31" t="s">
         <v>211</v>
       </c>
@@ -5457,7 +5465,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="183" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="31" t="s">
         <v>211</v>
       </c>
@@ -5477,7 +5485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="184" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="32" t="s">
         <v>218</v>
       </c>
@@ -5497,7 +5505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="32" t="s">
         <v>218</v>
       </c>
@@ -5517,7 +5525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="32" t="s">
         <v>218</v>
       </c>
@@ -5537,7 +5545,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="32" t="s">
         <v>218</v>
       </c>
@@ -5557,7 +5565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="32" t="s">
         <v>218</v>
       </c>
@@ -5577,7 +5585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="32" t="s">
         <v>218</v>
       </c>
@@ -5597,7 +5605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="32" t="s">
         <v>218</v>
       </c>
@@ -5617,7 +5625,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="32" t="s">
         <v>218</v>
       </c>
@@ -5637,7 +5645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="32" t="s">
         <v>218</v>
       </c>
@@ -5657,7 +5665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="32" t="s">
         <v>218</v>
       </c>
@@ -5677,7 +5685,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="194" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="32" t="s">
         <v>218</v>
       </c>
@@ -5697,7 +5705,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="32" t="s">
         <v>218</v>
       </c>
@@ -5717,7 +5725,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="32" t="s">
         <v>218</v>
       </c>
@@ -5737,7 +5745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="32" t="s">
         <v>218</v>
       </c>
@@ -5757,7 +5765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="32" t="s">
         <v>218</v>
       </c>
@@ -5777,7 +5785,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="32" t="s">
         <v>218</v>
       </c>
@@ -5797,7 +5805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="33" t="s">
         <v>235</v>
       </c>
@@ -5817,7 +5825,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="201" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="33" t="s">
         <v>235</v>
       </c>
@@ -5837,7 +5845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="202" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="33" t="s">
         <v>235</v>
       </c>
@@ -5857,7 +5865,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="33" t="s">
         <v>235</v>
       </c>
@@ -5877,7 +5885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="33" t="s">
         <v>235</v>
       </c>
@@ -5897,7 +5905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="33" t="s">
         <v>235</v>
       </c>
@@ -5917,7 +5925,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="33" t="s">
         <v>235</v>
       </c>
@@ -5937,7 +5945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="33" t="s">
         <v>235</v>
       </c>
@@ -5957,7 +5965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="33" t="s">
         <v>235</v>
       </c>
@@ -5977,7 +5985,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="33" t="s">
         <v>235</v>
       </c>
@@ -5997,7 +6005,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="32" t="s">
         <v>218</v>
       </c>
@@ -6017,7 +6025,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="32" t="s">
         <v>218</v>
       </c>
@@ -6037,7 +6045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="212" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="32" t="s">
         <v>218</v>
       </c>
@@ -6057,7 +6065,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="32" t="s">
         <v>218</v>
       </c>
@@ -6077,7 +6085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="32" t="s">
         <v>218</v>
       </c>
@@ -6097,7 +6105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="32" t="s">
         <v>218</v>
       </c>
@@ -6117,7 +6125,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="32" t="s">
         <v>218</v>
       </c>
@@ -6137,7 +6145,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="32" t="s">
         <v>218</v>
       </c>
@@ -6157,7 +6165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="32" t="s">
         <v>218</v>
       </c>
@@ -6177,7 +6185,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="32" t="s">
         <v>218</v>
       </c>
@@ -6197,7 +6205,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="220" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="32" t="s">
         <v>218</v>
       </c>
@@ -6217,7 +6225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="221" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="32" t="s">
         <v>218</v>
       </c>
@@ -6237,7 +6245,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="222" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="32" t="s">
         <v>218</v>
       </c>
@@ -6257,7 +6265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="33" t="s">
         <v>235</v>
       </c>
@@ -6277,7 +6285,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="33" t="s">
         <v>235</v>
       </c>
@@ -6297,7 +6305,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="225" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="33" t="s">
         <v>235</v>
       </c>
@@ -6317,7 +6325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="33" t="s">
         <v>235</v>
       </c>
@@ -6337,7 +6345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="227" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="33" t="s">
         <v>235</v>
       </c>
@@ -6357,7 +6365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="228" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="33" t="s">
         <v>235</v>
       </c>
@@ -6377,7 +6385,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="229" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="33" t="s">
         <v>235</v>
       </c>
@@ -6397,7 +6405,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="230" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="33" t="s">
         <v>235</v>
       </c>
@@ -6417,7 +6425,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="231" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="34" t="s">
         <v>267</v>
       </c>
@@ -6437,7 +6445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="232" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="34" t="s">
         <v>267</v>
       </c>
@@ -6457,7 +6465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="233" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="34" t="s">
         <v>267</v>
       </c>
@@ -6477,7 +6485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="34" t="s">
         <v>267</v>
       </c>
@@ -6497,7 +6505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="235" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="34" t="s">
         <v>267</v>
       </c>
@@ -6517,7 +6525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="236" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="34" t="s">
         <v>267</v>
       </c>
@@ -6537,7 +6545,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="237" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="34" t="s">
         <v>267</v>
       </c>
@@ -6557,7 +6565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="34" t="s">
         <v>267</v>
       </c>
@@ -6577,7 +6585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="239" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="34" t="s">
         <v>267</v>
       </c>
@@ -6597,7 +6605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="240" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="34" t="s">
         <v>267</v>
       </c>
@@ -6617,7 +6625,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="34" t="s">
         <v>267</v>
       </c>
@@ -6637,7 +6645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="34" t="s">
         <v>267</v>
       </c>
@@ -6657,7 +6665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="243" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="34" t="s">
         <v>267</v>
       </c>
@@ -6677,7 +6685,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="34" t="s">
         <v>267</v>
       </c>
@@ -6697,7 +6705,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="245" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A245" s="34" t="s">
         <v>267</v>
       </c>
@@ -6717,7 +6725,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="34" t="s">
         <v>267</v>
       </c>
@@ -6738,16 +6746,22 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F246"/>
+  <autoFilter ref="A1:F246" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="DEODORANTS (MEN)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -6756,7 +6770,7 @@
     <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
         <v>18</v>
       </c>
@@ -6773,7 +6787,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
         <v>24</v>
       </c>
@@ -6790,7 +6804,7 @@
         <v>7208</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>49</v>
       </c>
@@ -6807,7 +6821,7 @@
         <v>11186</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="44" t="s">
         <v>85</v>
       </c>
@@ -6824,7 +6838,7 @@
         <v>17200</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="48" t="s">
         <v>91</v>
       </c>
@@ -6841,7 +6855,7 @@
         <v>9556</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="52" t="s">
         <v>110</v>
       </c>
@@ -6858,7 +6872,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="56" t="s">
         <v>116</v>
       </c>
@@ -6875,7 +6889,7 @@
         <v>16800</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
         <v>122</v>
       </c>
@@ -6892,7 +6906,7 @@
         <v>24375</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="64" t="s">
         <v>135</v>
       </c>
@@ -6909,7 +6923,7 @@
         <v>38771</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="68" t="s">
         <v>195</v>
       </c>
@@ -6926,7 +6940,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="72" t="s">
         <v>200</v>
       </c>
@@ -6934,7 +6948,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="74">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="D11" s="75">
         <v>2000</v>
@@ -6943,7 +6957,7 @@
         <v>15300</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
         <v>206</v>
       </c>
@@ -6960,7 +6974,7 @@
         <v>2750</v>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="56" t="s">
         <v>211</v>
       </c>
@@ -6977,7 +6991,7 @@
         <v>2317</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="76" t="s">
         <v>218</v>
       </c>
@@ -6994,7 +7008,7 @@
         <v>7563</v>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
         <v>235</v>
       </c>
@@ -7013,6 +7027,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: sync spreadsheet Current Price column to reflect live prices
Updated Current Price (XAF) for all 251 products in AmericanSelect_PricingAnalysis.xlsx
to match the prices now live in categories.ts. Current = Suggested for all items.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis.xlsx
+++ b/AmericanSelect_PricingAnalysis.xlsx
@@ -530,7 +530,7 @@
         <v>5.87</v>
       </c>
       <c r="D2">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E2">
         <v>7000</v>
@@ -562,7 +562,7 @@
         <v>5.87</v>
       </c>
       <c r="D3">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E3">
         <v>7000</v>
@@ -594,7 +594,7 @@
         <v>5.87</v>
       </c>
       <c r="D4">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E4">
         <v>7000</v>
@@ -626,7 +626,7 @@
         <v>5.87</v>
       </c>
       <c r="D5">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E5">
         <v>7000</v>
@@ -658,7 +658,7 @@
         <v>5.87</v>
       </c>
       <c r="D6">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E6">
         <v>7000</v>
@@ -690,7 +690,7 @@
         <v>5.87</v>
       </c>
       <c r="D7">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E7">
         <v>7000</v>
@@ -722,7 +722,7 @@
         <v>5.87</v>
       </c>
       <c r="D8">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E8">
         <v>7000</v>
@@ -754,7 +754,7 @@
         <v>7</v>
       </c>
       <c r="D9">
-        <v>3500</v>
+        <v>8500</v>
       </c>
       <c r="E9">
         <v>8500</v>
@@ -786,7 +786,7 @@
         <v>7</v>
       </c>
       <c r="D10">
-        <v>3500</v>
+        <v>8500</v>
       </c>
       <c r="E10">
         <v>8500</v>
@@ -818,7 +818,7 @@
         <v>7</v>
       </c>
       <c r="D11">
-        <v>3500</v>
+        <v>8500</v>
       </c>
       <c r="E11">
         <v>8500</v>
@@ -850,7 +850,7 @@
         <v>2.97</v>
       </c>
       <c r="D12">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E12">
         <v>4500</v>
@@ -882,7 +882,7 @@
         <v>2.97</v>
       </c>
       <c r="D13">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E13">
         <v>4500</v>
@@ -914,7 +914,7 @@
         <v>4.68</v>
       </c>
       <c r="D14">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E14">
         <v>7000</v>
@@ -946,7 +946,7 @@
         <v>2.97</v>
       </c>
       <c r="D15">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E15">
         <v>4500</v>
@@ -978,7 +978,7 @@
         <v>2.97</v>
       </c>
       <c r="D16">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E16">
         <v>4500</v>
@@ -1010,7 +1010,7 @@
         <v>4.68</v>
       </c>
       <c r="D17">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E17">
         <v>7000</v>
@@ -1042,7 +1042,7 @@
         <v>4.68</v>
       </c>
       <c r="D18">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E18">
         <v>7000</v>
@@ -1074,7 +1074,7 @@
         <v>4.68</v>
       </c>
       <c r="D19">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E19">
         <v>7000</v>
@@ -1106,7 +1106,7 @@
         <v>4.68</v>
       </c>
       <c r="D20">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E20">
         <v>7000</v>
@@ -1138,7 +1138,7 @@
         <v>6.5</v>
       </c>
       <c r="D21">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="E21">
         <v>5000</v>
@@ -1170,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="D22">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="E22">
         <v>1500</v>
@@ -1202,7 +1202,7 @@
         <v>4.5</v>
       </c>
       <c r="D23">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="E23">
         <v>5000</v>
@@ -1234,7 +1234,7 @@
         <v>4.5</v>
       </c>
       <c r="D24">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="E24">
         <v>5000</v>
@@ -1266,7 +1266,7 @@
         <v>4.5</v>
       </c>
       <c r="D25">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="E25">
         <v>5000</v>
@@ -1298,7 +1298,7 @@
         <v>10</v>
       </c>
       <c r="D26">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E26">
         <v>15000</v>
@@ -1330,7 +1330,7 @@
         <v>10</v>
       </c>
       <c r="D27">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E27">
         <v>15000</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="D28">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E28">
         <v>15000</v>
@@ -1394,7 +1394,7 @@
         <v>10</v>
       </c>
       <c r="D29">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E29">
         <v>15000</v>
@@ -1426,7 +1426,7 @@
         <v>9</v>
       </c>
       <c r="D30">
-        <v>6000</v>
+        <v>12300</v>
       </c>
       <c r="E30">
         <v>14000</v>
@@ -1458,7 +1458,7 @@
         <v>6</v>
       </c>
       <c r="D31">
-        <v>6500</v>
+        <v>10500</v>
       </c>
       <c r="E31">
         <v>10500</v>
@@ -1490,7 +1490,7 @@
         <v>6</v>
       </c>
       <c r="D32">
-        <v>6500</v>
+        <v>10500</v>
       </c>
       <c r="E32">
         <v>10500</v>
@@ -1522,7 +1522,7 @@
         <v>6</v>
       </c>
       <c r="D33">
-        <v>6500</v>
+        <v>10500</v>
       </c>
       <c r="E33">
         <v>10500</v>
@@ -1554,7 +1554,7 @@
         <v>6</v>
       </c>
       <c r="D34">
-        <v>6500</v>
+        <v>10500</v>
       </c>
       <c r="E34">
         <v>10500</v>
@@ -1586,7 +1586,7 @@
         <v>6</v>
       </c>
       <c r="D35">
-        <v>6500</v>
+        <v>10500</v>
       </c>
       <c r="E35">
         <v>10500</v>
@@ -1618,7 +1618,7 @@
         <v>6</v>
       </c>
       <c r="D36">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E36">
         <v>11500</v>
@@ -1650,7 +1650,7 @@
         <v>6</v>
       </c>
       <c r="D37">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E37">
         <v>11500</v>
@@ -1682,7 +1682,7 @@
         <v>6</v>
       </c>
       <c r="D38">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E38">
         <v>11500</v>
@@ -1714,7 +1714,7 @@
         <v>6</v>
       </c>
       <c r="D39">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E39">
         <v>11500</v>
@@ -1746,7 +1746,7 @@
         <v>6</v>
       </c>
       <c r="D40">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E40">
         <v>11500</v>
@@ -1778,7 +1778,7 @@
         <v>6</v>
       </c>
       <c r="D41">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="E41">
         <v>11500</v>
@@ -1810,7 +1810,7 @@
         <v>6</v>
       </c>
       <c r="D42">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E42">
         <v>8000</v>
@@ -1842,7 +1842,7 @@
         <v>6</v>
       </c>
       <c r="D43">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E43">
         <v>8000</v>
@@ -1874,7 +1874,7 @@
         <v>6</v>
       </c>
       <c r="D44">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E44">
         <v>8000</v>
@@ -1906,7 +1906,7 @@
         <v>6</v>
       </c>
       <c r="D45">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E45">
         <v>8000</v>
@@ -1938,7 +1938,7 @@
         <v>6</v>
       </c>
       <c r="D46">
-        <v>6500</v>
+        <v>8500</v>
       </c>
       <c r="E46">
         <v>8500</v>
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D47">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E47">
         <v>8000</v>
@@ -2002,7 +2002,7 @@
         <v>6</v>
       </c>
       <c r="D48">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E48">
         <v>8000</v>
@@ -2034,7 +2034,7 @@
         <v>6</v>
       </c>
       <c r="D49">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E49">
         <v>8000</v>
@@ -2066,7 +2066,7 @@
         <v>6</v>
       </c>
       <c r="D50">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E50">
         <v>8000</v>
@@ -2098,7 +2098,7 @@
         <v>6</v>
       </c>
       <c r="D51">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E51">
         <v>8000</v>
@@ -2130,7 +2130,7 @@
         <v>6</v>
       </c>
       <c r="D52">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E52">
         <v>8000</v>
@@ -2162,7 +2162,7 @@
         <v>6</v>
       </c>
       <c r="D53">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E53">
         <v>8000</v>
@@ -2194,7 +2194,7 @@
         <v>6</v>
       </c>
       <c r="D54">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E54">
         <v>8000</v>
@@ -2226,7 +2226,7 @@
         <v>6</v>
       </c>
       <c r="D55">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E55">
         <v>8000</v>
@@ -2258,7 +2258,7 @@
         <v>13</v>
       </c>
       <c r="D56">
-        <v>10000</v>
+        <v>16500</v>
       </c>
       <c r="E56">
         <v>16500</v>
@@ -2290,7 +2290,7 @@
         <v>15</v>
       </c>
       <c r="D57">
-        <v>10000</v>
+        <v>17000</v>
       </c>
       <c r="E57">
         <v>17000</v>
@@ -2322,7 +2322,7 @@
         <v>20</v>
       </c>
       <c r="D58">
-        <v>10000</v>
+        <v>17000</v>
       </c>
       <c r="E58">
         <v>17000</v>
@@ -2354,7 +2354,7 @@
         <v>10</v>
       </c>
       <c r="D59">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E59">
         <v>15000</v>
@@ -2386,7 +2386,7 @@
         <v>4</v>
       </c>
       <c r="D60">
-        <v>3500</v>
+        <v>8000</v>
       </c>
       <c r="E60">
         <v>8000</v>
@@ -2418,7 +2418,7 @@
         <v>2.5</v>
       </c>
       <c r="D61">
-        <v>1500</v>
+        <v>2800</v>
       </c>
       <c r="E61">
         <v>3500</v>
@@ -2450,7 +2450,7 @@
         <v>6</v>
       </c>
       <c r="D62">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E62">
         <v>10000</v>
@@ -2482,7 +2482,7 @@
         <v>9</v>
       </c>
       <c r="D63">
-        <v>4500</v>
+        <v>8000</v>
       </c>
       <c r="E63">
         <v>8000</v>
@@ -2514,7 +2514,7 @@
         <v>18</v>
       </c>
       <c r="D64">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E64">
         <v>20000</v>
@@ -2546,7 +2546,7 @@
         <v>22</v>
       </c>
       <c r="D65">
-        <v>12000</v>
+        <v>18900</v>
       </c>
       <c r="E65">
         <v>18900</v>
@@ -2578,7 +2578,7 @@
         <v>6</v>
       </c>
       <c r="D66">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="E66">
         <v>13000</v>
@@ -2610,7 +2610,7 @@
         <v>6</v>
       </c>
       <c r="D67">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="E67">
         <v>13000</v>
@@ -2642,7 +2642,7 @@
         <v>11</v>
       </c>
       <c r="D68">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E68">
         <v>15000</v>
@@ -2674,7 +2674,7 @@
         <v>11</v>
       </c>
       <c r="D69">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E69">
         <v>15000</v>
@@ -2706,7 +2706,7 @@
         <v>11</v>
       </c>
       <c r="D70">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E70">
         <v>15000</v>
@@ -2738,7 +2738,7 @@
         <v>11</v>
       </c>
       <c r="D71">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E71">
         <v>15000</v>
@@ -2770,7 +2770,7 @@
         <v>11</v>
       </c>
       <c r="D72">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E72">
         <v>15000</v>
@@ -2802,7 +2802,7 @@
         <v>4.5</v>
       </c>
       <c r="D73">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E73">
         <v>7000</v>
@@ -2834,7 +2834,7 @@
         <v>4.5</v>
       </c>
       <c r="D74">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E74">
         <v>7000</v>
@@ -2866,7 +2866,7 @@
         <v>4.5</v>
       </c>
       <c r="D75">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E75">
         <v>7000</v>
@@ -2898,7 +2898,7 @@
         <v>4.5</v>
       </c>
       <c r="D76">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E76">
         <v>7000</v>
@@ -2930,7 +2930,7 @@
         <v>4.5</v>
       </c>
       <c r="D77">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E77">
         <v>7000</v>
@@ -2962,7 +2962,7 @@
         <v>4.5</v>
       </c>
       <c r="D78">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E78">
         <v>7000</v>
@@ -2994,7 +2994,7 @@
         <v>4.5</v>
       </c>
       <c r="D79">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E79">
         <v>7000</v>
@@ -3026,7 +3026,7 @@
         <v>4.5</v>
       </c>
       <c r="D80">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E80">
         <v>7000</v>
@@ -3058,7 +3058,7 @@
         <v>4.5</v>
       </c>
       <c r="D81">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E81">
         <v>7000</v>
@@ -3090,7 +3090,7 @@
         <v>4.5</v>
       </c>
       <c r="D82">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E82">
         <v>7000</v>
@@ -3122,7 +3122,7 @@
         <v>4.5</v>
       </c>
       <c r="D83">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="E83">
         <v>7000</v>
@@ -3154,7 +3154,7 @@
         <v>6</v>
       </c>
       <c r="D84">
-        <v>4500</v>
+        <v>9000</v>
       </c>
       <c r="E84">
         <v>9000</v>
@@ -3186,7 +3186,7 @@
         <v>6</v>
       </c>
       <c r="D85">
-        <v>4500</v>
+        <v>9000</v>
       </c>
       <c r="E85">
         <v>9000</v>
@@ -3218,7 +3218,7 @@
         <v>4</v>
       </c>
       <c r="D86">
-        <v>4500</v>
+        <v>6000</v>
       </c>
       <c r="E86">
         <v>6000</v>
@@ -3250,7 +3250,7 @@
         <v>10</v>
       </c>
       <c r="D87">
-        <v>8500</v>
+        <v>9500</v>
       </c>
       <c r="E87">
         <v>9500</v>
@@ -3282,7 +3282,7 @@
         <v>14</v>
       </c>
       <c r="D88">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E88">
         <v>10000</v>
@@ -3314,7 +3314,7 @@
         <v>3.97</v>
       </c>
       <c r="D89">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E89">
         <v>4000</v>
@@ -3346,7 +3346,7 @@
         <v>3.97</v>
       </c>
       <c r="D90">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E90">
         <v>4000</v>
@@ -3378,7 +3378,7 @@
         <v>3.97</v>
       </c>
       <c r="D91">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E91">
         <v>4000</v>
@@ -3410,7 +3410,7 @@
         <v>3.97</v>
       </c>
       <c r="D92">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E92">
         <v>4000</v>
@@ -3442,7 +3442,7 @@
         <v>40</v>
       </c>
       <c r="D93">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E93">
         <v>20000</v>
@@ -3474,7 +3474,7 @@
         <v>30</v>
       </c>
       <c r="D94">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="E94">
         <v>30000</v>
@@ -3506,7 +3506,7 @@
         <v>7</v>
       </c>
       <c r="D95">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E95">
         <v>3000</v>
@@ -3538,7 +3538,7 @@
         <v>10</v>
       </c>
       <c r="D96">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E96">
         <v>5000</v>
@@ -3570,7 +3570,7 @@
         <v>12</v>
       </c>
       <c r="D97">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E97">
         <v>10000</v>
@@ -3634,7 +3634,7 @@
         <v>20</v>
       </c>
       <c r="D99">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E99">
         <v>10000</v>
@@ -3666,7 +3666,7 @@
         <v>20</v>
       </c>
       <c r="D100">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E100">
         <v>10000</v>
@@ -3698,7 +3698,7 @@
         <v>20</v>
       </c>
       <c r="D101">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E101">
         <v>10000</v>
@@ -3730,7 +3730,7 @@
         <v>20</v>
       </c>
       <c r="D102">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E102">
         <v>10000</v>
@@ -3762,7 +3762,7 @@
         <v>20</v>
       </c>
       <c r="D103">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E103">
         <v>10000</v>
@@ -3922,7 +3922,7 @@
         <v>35</v>
       </c>
       <c r="D108">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E108">
         <v>15000</v>
@@ -3954,7 +3954,7 @@
         <v>35</v>
       </c>
       <c r="D109">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E109">
         <v>15000</v>
@@ -3986,7 +3986,7 @@
         <v>35</v>
       </c>
       <c r="D110">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E110">
         <v>15000</v>
@@ -4018,7 +4018,7 @@
         <v>35</v>
       </c>
       <c r="D111">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E111">
         <v>15000</v>
@@ -4050,7 +4050,7 @@
         <v>35</v>
       </c>
       <c r="D112">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E112">
         <v>15000</v>
@@ -4082,7 +4082,7 @@
         <v>35</v>
       </c>
       <c r="D113">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E113">
         <v>15000</v>
@@ -4114,7 +4114,7 @@
         <v>35</v>
       </c>
       <c r="D114">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E114">
         <v>15000</v>
@@ -4146,7 +4146,7 @@
         <v>38</v>
       </c>
       <c r="D115">
-        <v>9000</v>
+        <v>15000</v>
       </c>
       <c r="E115">
         <v>15000</v>
@@ -4178,7 +4178,7 @@
         <v>38</v>
       </c>
       <c r="D116">
-        <v>9000</v>
+        <v>15000</v>
       </c>
       <c r="E116">
         <v>15000</v>
@@ -4210,7 +4210,7 @@
         <v>35</v>
       </c>
       <c r="D117">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E117">
         <v>15000</v>
@@ -4242,7 +4242,7 @@
         <v>35</v>
       </c>
       <c r="D118">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="E118">
         <v>15000</v>
@@ -4274,7 +4274,7 @@
         <v>25</v>
       </c>
       <c r="D119">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="E119">
         <v>10000</v>
@@ -4306,7 +4306,7 @@
         <v>25</v>
       </c>
       <c r="D120">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="E120">
         <v>10000</v>
@@ -4338,7 +4338,7 @@
         <v>18</v>
       </c>
       <c r="D121">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E121">
         <v>10000</v>
@@ -4370,7 +4370,7 @@
         <v>28</v>
       </c>
       <c r="D122">
-        <v>7000</v>
+        <v>8900</v>
       </c>
       <c r="E122">
         <v>8900</v>
@@ -4402,7 +4402,7 @@
         <v>12</v>
       </c>
       <c r="D123">
-        <v>2500</v>
+        <v>7500</v>
       </c>
       <c r="E123">
         <v>7500</v>
@@ -4434,7 +4434,7 @@
         <v>18</v>
       </c>
       <c r="D124">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E124">
         <v>5000</v>
@@ -4466,7 +4466,7 @@
         <v>18</v>
       </c>
       <c r="D125">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E125">
         <v>5000</v>
@@ -4498,7 +4498,7 @@
         <v>18</v>
       </c>
       <c r="D126">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E126">
         <v>5000</v>
@@ -4530,7 +4530,7 @@
         <v>18</v>
       </c>
       <c r="D127">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E127">
         <v>5000</v>
@@ -4562,7 +4562,7 @@
         <v>18</v>
       </c>
       <c r="D128">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E128">
         <v>5000</v>
@@ -4594,7 +4594,7 @@
         <v>18</v>
       </c>
       <c r="D129">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E129">
         <v>15000</v>
@@ -4914,7 +4914,7 @@
         <v>15</v>
       </c>
       <c r="D139">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E139">
         <v>10000</v>
@@ -4946,7 +4946,7 @@
         <v>15</v>
       </c>
       <c r="D140">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E140">
         <v>10000</v>
@@ -4978,7 +4978,7 @@
         <v>15</v>
       </c>
       <c r="D141">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E141">
         <v>10000</v>
@@ -5010,7 +5010,7 @@
         <v>15</v>
       </c>
       <c r="D142">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E142">
         <v>10000</v>
@@ -5042,7 +5042,7 @@
         <v>25</v>
       </c>
       <c r="D143">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="E143">
         <v>10000</v>
@@ -5074,7 +5074,7 @@
         <v>25</v>
       </c>
       <c r="D144">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="E144">
         <v>10000</v>
@@ -5106,7 +5106,7 @@
         <v>25</v>
       </c>
       <c r="D145">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="E145">
         <v>10000</v>
@@ -5138,7 +5138,7 @@
         <v>30</v>
       </c>
       <c r="D146">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="E146">
         <v>10000</v>
@@ -5170,7 +5170,7 @@
         <v>30</v>
       </c>
       <c r="D147">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="E147">
         <v>7000</v>
@@ -5202,7 +5202,7 @@
         <v>18</v>
       </c>
       <c r="D148">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E148">
         <v>10000</v>
@@ -5234,7 +5234,7 @@
         <v>25</v>
       </c>
       <c r="D149">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E149">
         <v>25000</v>
@@ -5266,7 +5266,7 @@
         <v>28</v>
       </c>
       <c r="D150">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E150">
         <v>10000</v>
@@ -5298,7 +5298,7 @@
         <v>32</v>
       </c>
       <c r="D151">
-        <v>5500</v>
+        <v>10000</v>
       </c>
       <c r="E151">
         <v>10000</v>
@@ -5330,7 +5330,7 @@
         <v>32</v>
       </c>
       <c r="D152">
-        <v>5500</v>
+        <v>10000</v>
       </c>
       <c r="E152">
         <v>10000</v>
@@ -5362,7 +5362,7 @@
         <v>32</v>
       </c>
       <c r="D153">
-        <v>5500</v>
+        <v>10000</v>
       </c>
       <c r="E153">
         <v>10000</v>
@@ -5394,7 +5394,7 @@
         <v>32</v>
       </c>
       <c r="D154">
-        <v>5500</v>
+        <v>10000</v>
       </c>
       <c r="E154">
         <v>10000</v>
@@ -5426,7 +5426,7 @@
         <v>32</v>
       </c>
       <c r="D155">
-        <v>5500</v>
+        <v>10000</v>
       </c>
       <c r="E155">
         <v>10000</v>
@@ -5522,7 +5522,7 @@
         <v>25</v>
       </c>
       <c r="D158">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="E158">
         <v>10000</v>
@@ -5554,7 +5554,7 @@
         <v>25</v>
       </c>
       <c r="D159">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="E159">
         <v>10000</v>
@@ -5586,7 +5586,7 @@
         <v>32</v>
       </c>
       <c r="D160">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="E160">
         <v>10000</v>
@@ -5618,7 +5618,7 @@
         <v>30</v>
       </c>
       <c r="D161">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E161">
         <v>10000</v>
@@ -5650,7 +5650,7 @@
         <v>7</v>
       </c>
       <c r="D162">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E162">
         <v>5000</v>
@@ -5682,7 +5682,7 @@
         <v>12</v>
       </c>
       <c r="D163">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="E163">
         <v>5000</v>
@@ -5714,7 +5714,7 @@
         <v>20</v>
       </c>
       <c r="D164">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E164">
         <v>8000</v>
@@ -5746,7 +5746,7 @@
         <v>20</v>
       </c>
       <c r="D165">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="E165">
         <v>10000</v>
@@ -5778,7 +5778,7 @@
         <v>32</v>
       </c>
       <c r="D166">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E166">
         <v>25000</v>
@@ -5810,7 +5810,7 @@
         <v>40</v>
       </c>
       <c r="D167">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E167">
         <v>25000</v>
@@ -5842,7 +5842,7 @@
         <v>20</v>
       </c>
       <c r="D168">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E168">
         <v>20000</v>
@@ -5874,7 +5874,7 @@
         <v>7</v>
       </c>
       <c r="D169">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="E169">
         <v>2500</v>
@@ -5906,7 +5906,7 @@
         <v>7</v>
       </c>
       <c r="D170">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="E170">
         <v>2500</v>
@@ -5938,7 +5938,7 @@
         <v>7</v>
       </c>
       <c r="D171">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="E171">
         <v>2500</v>
@@ -6034,7 +6034,7 @@
         <v>4.5</v>
       </c>
       <c r="D174">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="E174">
         <v>6000</v>
@@ -6066,7 +6066,7 @@
         <v>5</v>
       </c>
       <c r="D175">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="E175">
         <v>6000</v>
@@ -6098,7 +6098,7 @@
         <v>5</v>
       </c>
       <c r="D176">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="E176">
         <v>6000</v>
@@ -6130,7 +6130,7 @@
         <v>4</v>
       </c>
       <c r="D177">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E177">
         <v>6000</v>
@@ -6162,7 +6162,7 @@
         <v>3.5</v>
       </c>
       <c r="D178">
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="E178">
         <v>5500</v>
@@ -6194,7 +6194,7 @@
         <v>3</v>
       </c>
       <c r="D179">
-        <v>2300</v>
+        <v>5500</v>
       </c>
       <c r="E179">
         <v>5500</v>
@@ -6226,7 +6226,7 @@
         <v>3</v>
       </c>
       <c r="D180">
-        <v>2300</v>
+        <v>5500</v>
       </c>
       <c r="E180">
         <v>5500</v>
@@ -6258,7 +6258,7 @@
         <v>3</v>
       </c>
       <c r="D181">
-        <v>2300</v>
+        <v>5500</v>
       </c>
       <c r="E181">
         <v>5500</v>
@@ -6290,7 +6290,7 @@
         <v>3</v>
       </c>
       <c r="D182">
-        <v>2300</v>
+        <v>5500</v>
       </c>
       <c r="E182">
         <v>5500</v>
@@ -6322,7 +6322,7 @@
         <v>4.5</v>
       </c>
       <c r="D183">
-        <v>3200</v>
+        <v>5500</v>
       </c>
       <c r="E183">
         <v>5500</v>
@@ -6354,7 +6354,7 @@
         <v>15</v>
       </c>
       <c r="D184">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="E184">
         <v>15000</v>
@@ -6386,7 +6386,7 @@
         <v>15</v>
       </c>
       <c r="D185">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="E185">
         <v>15000</v>
@@ -6418,7 +6418,7 @@
         <v>12</v>
       </c>
       <c r="D186">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="E186">
         <v>13000</v>
@@ -6514,7 +6514,7 @@
         <v>12</v>
       </c>
       <c r="D189">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="E189">
         <v>13000</v>
@@ -6546,7 +6546,7 @@
         <v>12</v>
       </c>
       <c r="D190">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="E190">
         <v>13000</v>
@@ -6578,7 +6578,7 @@
         <v>10</v>
       </c>
       <c r="D191">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E191">
         <v>8000</v>
@@ -6610,7 +6610,7 @@
         <v>10</v>
       </c>
       <c r="D192">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="E192">
         <v>8000</v>
@@ -6642,7 +6642,7 @@
         <v>8</v>
       </c>
       <c r="D193">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E193">
         <v>8000</v>
@@ -6674,7 +6674,7 @@
         <v>8</v>
       </c>
       <c r="D194">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E194">
         <v>8000</v>
@@ -6706,7 +6706,7 @@
         <v>8</v>
       </c>
       <c r="D195">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E195">
         <v>7000</v>
@@ -6738,7 +6738,7 @@
         <v>8</v>
       </c>
       <c r="D196">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E196">
         <v>7000</v>
@@ -6770,7 +6770,7 @@
         <v>8</v>
       </c>
       <c r="D197">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E197">
         <v>7000</v>
@@ -6802,7 +6802,7 @@
         <v>8</v>
       </c>
       <c r="D198">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E198">
         <v>7000</v>
@@ -6834,7 +6834,7 @@
         <v>5</v>
       </c>
       <c r="D199">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="E199">
         <v>7000</v>
@@ -6866,7 +6866,7 @@
         <v>12</v>
       </c>
       <c r="D200">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E200">
         <v>15000</v>
@@ -6898,7 +6898,7 @@
         <v>12</v>
       </c>
       <c r="D201">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E201">
         <v>15000</v>
@@ -6930,7 +6930,7 @@
         <v>12</v>
       </c>
       <c r="D202">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E202">
         <v>15000</v>
@@ -6962,7 +6962,7 @@
         <v>12</v>
       </c>
       <c r="D203">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E203">
         <v>15000</v>
@@ -6994,7 +6994,7 @@
         <v>12</v>
       </c>
       <c r="D204">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E204">
         <v>15000</v>
@@ -7026,7 +7026,7 @@
         <v>12</v>
       </c>
       <c r="D205">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E205">
         <v>15000</v>
@@ -7058,7 +7058,7 @@
         <v>12</v>
       </c>
       <c r="D206">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E206">
         <v>15000</v>
@@ -7090,7 +7090,7 @@
         <v>12</v>
       </c>
       <c r="D207">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E207">
         <v>15000</v>
@@ -7122,7 +7122,7 @@
         <v>12</v>
       </c>
       <c r="D208">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E208">
         <v>15000</v>
@@ -7154,7 +7154,7 @@
         <v>8</v>
       </c>
       <c r="D209">
-        <v>6500</v>
+        <v>9000</v>
       </c>
       <c r="E209">
         <v>9000</v>
@@ -7186,7 +7186,7 @@
         <v>5</v>
       </c>
       <c r="D210">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E210">
         <v>7000</v>
@@ -7218,7 +7218,7 @@
         <v>5</v>
       </c>
       <c r="D211">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E211">
         <v>7000</v>
@@ -7250,7 +7250,7 @@
         <v>5</v>
       </c>
       <c r="D212">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E212">
         <v>7000</v>
@@ -7282,7 +7282,7 @@
         <v>5</v>
       </c>
       <c r="D213">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E213">
         <v>7000</v>
@@ -7314,7 +7314,7 @@
         <v>5</v>
       </c>
       <c r="D214">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E214">
         <v>7000</v>
@@ -7346,7 +7346,7 @@
         <v>5</v>
       </c>
       <c r="D215">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="E215">
         <v>7000</v>
@@ -7378,7 +7378,7 @@
         <v>10</v>
       </c>
       <c r="D216">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="E216">
         <v>7000</v>
@@ -7410,7 +7410,7 @@
         <v>15</v>
       </c>
       <c r="D217">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E217">
         <v>17500</v>
@@ -7442,7 +7442,7 @@
         <v>15</v>
       </c>
       <c r="D218">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E218">
         <v>17500</v>
@@ -7474,7 +7474,7 @@
         <v>15</v>
       </c>
       <c r="D219">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E219">
         <v>17500</v>
@@ -7506,7 +7506,7 @@
         <v>15</v>
       </c>
       <c r="D220">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E220">
         <v>17500</v>
@@ -7538,7 +7538,7 @@
         <v>15</v>
       </c>
       <c r="D221">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E221">
         <v>17500</v>
@@ -7570,7 +7570,7 @@
         <v>15</v>
       </c>
       <c r="D222">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E222">
         <v>17500</v>
@@ -7602,7 +7602,7 @@
         <v>5</v>
       </c>
       <c r="D223">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E223">
         <v>8000</v>
@@ -7634,7 +7634,7 @@
         <v>8</v>
       </c>
       <c r="D224">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E224">
         <v>10000</v>
@@ -7666,7 +7666,7 @@
         <v>8</v>
       </c>
       <c r="D225">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E225">
         <v>10000</v>
@@ -7698,7 +7698,7 @@
         <v>8</v>
       </c>
       <c r="D226">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E226">
         <v>10000</v>
@@ -7730,7 +7730,7 @@
         <v>5</v>
       </c>
       <c r="D227">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E227">
         <v>8000</v>
@@ -7762,7 +7762,7 @@
         <v>10</v>
       </c>
       <c r="D228">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="E228">
         <v>12000</v>
@@ -7826,7 +7826,7 @@
         <v>15</v>
       </c>
       <c r="D230">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="E230">
         <v>17500</v>
@@ -7858,7 +7858,7 @@
         <v>3</v>
       </c>
       <c r="D231">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E231">
         <v>4500</v>
@@ -7890,7 +7890,7 @@
         <v>3</v>
       </c>
       <c r="D232">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E232">
         <v>4500</v>
@@ -7922,7 +7922,7 @@
         <v>3</v>
       </c>
       <c r="D233">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E233">
         <v>4500</v>
@@ -7954,7 +7954,7 @@
         <v>3</v>
       </c>
       <c r="D234">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E234">
         <v>4500</v>
@@ -7986,7 +7986,7 @@
         <v>3</v>
       </c>
       <c r="D235">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E235">
         <v>4500</v>
@@ -8018,7 +8018,7 @@
         <v>3</v>
       </c>
       <c r="D236">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E236">
         <v>4500</v>
@@ -8050,7 +8050,7 @@
         <v>3</v>
       </c>
       <c r="D237">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E237">
         <v>4500</v>
@@ -8082,7 +8082,7 @@
         <v>3</v>
       </c>
       <c r="D238">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E238">
         <v>4500</v>
@@ -8114,7 +8114,7 @@
         <v>3</v>
       </c>
       <c r="D239">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E239">
         <v>4500</v>
@@ -8146,7 +8146,7 @@
         <v>3</v>
       </c>
       <c r="D240">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E240">
         <v>4500</v>
@@ -8178,7 +8178,7 @@
         <v>3</v>
       </c>
       <c r="D241">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E241">
         <v>4500</v>
@@ -8210,7 +8210,7 @@
         <v>3</v>
       </c>
       <c r="D242">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E242">
         <v>4500</v>
@@ -8242,7 +8242,7 @@
         <v>3</v>
       </c>
       <c r="D243">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E243">
         <v>4500</v>
@@ -8274,7 +8274,7 @@
         <v>3</v>
       </c>
       <c r="D244">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E244">
         <v>4500</v>
@@ -8306,7 +8306,7 @@
         <v>3</v>
       </c>
       <c r="D245">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E245">
         <v>4500</v>
@@ -8338,7 +8338,7 @@
         <v>3</v>
       </c>
       <c r="D246">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E246">
         <v>4500</v>
@@ -8369,8 +8369,8 @@
       <c r="C247" t="str">
         <v/>
       </c>
-      <c r="D247" t="str">
-        <v/>
+      <c r="D247">
+        <v>5000</v>
       </c>
       <c r="E247">
         <v>5000</v>
@@ -8401,8 +8401,8 @@
       <c r="C248" t="str">
         <v/>
       </c>
-      <c r="D248" t="str">
-        <v/>
+      <c r="D248">
+        <v>35000</v>
       </c>
       <c r="E248">
         <v>35000</v>
@@ -8433,8 +8433,8 @@
       <c r="C249" t="str">
         <v/>
       </c>
-      <c r="D249" t="str">
-        <v/>
+      <c r="D249">
+        <v>3500</v>
       </c>
       <c r="E249">
         <v>3500</v>
@@ -8465,8 +8465,8 @@
       <c r="C250" t="str">
         <v/>
       </c>
-      <c r="D250" t="str">
-        <v/>
+      <c r="D250">
+        <v>3000</v>
       </c>
       <c r="E250">
         <v>3000</v>
@@ -8497,8 +8497,8 @@
       <c r="C251" t="str">
         <v/>
       </c>
-      <c r="D251" t="str">
-        <v/>
+      <c r="D251">
+        <v>2500</v>
       </c>
       <c r="E251">
         <v>2500</v>
@@ -8558,7 +8558,7 @@
         <v>4.93</v>
       </c>
       <c r="D2">
-        <v>4200</v>
+        <v>6208</v>
       </c>
       <c r="E2">
         <v>6208</v>
@@ -8575,7 +8575,7 @@
         <v>7.46</v>
       </c>
       <c r="D3">
-        <v>6857</v>
+        <v>10851</v>
       </c>
       <c r="E3">
         <v>10900</v>
@@ -8592,7 +8592,7 @@
         <v>11.5</v>
       </c>
       <c r="D4">
-        <v>7400</v>
+        <v>11940</v>
       </c>
       <c r="E4">
         <v>12080</v>
@@ -8609,7 +8609,7 @@
         <v>6.47</v>
       </c>
       <c r="D5">
-        <v>6639</v>
+        <v>9889</v>
       </c>
       <c r="E5">
         <v>9889</v>
@@ -8626,7 +8626,7 @@
         <v>8</v>
       </c>
       <c r="D6">
-        <v>6000</v>
+        <v>8700</v>
       </c>
       <c r="E6">
         <v>8700</v>
@@ -8643,7 +8643,7 @@
         <v>7.98</v>
       </c>
       <c r="D7">
-        <v>3286</v>
+        <v>10857</v>
       </c>
       <c r="E7">
         <v>10857</v>
@@ -8660,7 +8660,7 @@
         <v>13</v>
       </c>
       <c r="D8">
-        <v>6533</v>
+        <v>8800</v>
       </c>
       <c r="E8">
         <v>9200</v>
@@ -8677,7 +8677,7 @@
         <v>25.85</v>
       </c>
       <c r="D9">
-        <v>7051</v>
+        <v>10414</v>
       </c>
       <c r="E9">
         <v>11220</v>
@@ -8694,7 +8694,7 @@
         <v>28</v>
       </c>
       <c r="D10">
-        <v>10750</v>
+        <v>20000</v>
       </c>
       <c r="E10">
         <v>20000</v>
@@ -8711,7 +8711,7 @@
         <v>10.2</v>
       </c>
       <c r="D11">
-        <v>2000</v>
+        <v>2900</v>
       </c>
       <c r="E11">
         <v>3500</v>
@@ -8728,7 +8728,7 @@
         <v>4.63</v>
       </c>
       <c r="D12">
-        <v>2750</v>
+        <v>6000</v>
       </c>
       <c r="E12">
         <v>6000</v>
@@ -8745,7 +8745,7 @@
         <v>3.33</v>
       </c>
       <c r="D13">
-        <v>2317</v>
+        <v>5500</v>
       </c>
       <c r="E13">
         <v>5500</v>
@@ -8762,7 +8762,7 @@
         <v>10.1</v>
       </c>
       <c r="D14">
-        <v>8655</v>
+        <v>10690</v>
       </c>
       <c r="E14">
         <v>10897</v>
@@ -8779,7 +8779,7 @@
         <v>10.17</v>
       </c>
       <c r="D15">
-        <v>9083</v>
+        <v>12639</v>
       </c>
       <c r="E15">
         <v>12639</v>
@@ -8796,7 +8796,7 @@
         <v>3</v>
       </c>
       <c r="D16">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="E16">
         <v>4500</v>

</xml_diff>